<commit_message>
update indicator library forest
Former-commit-id: af58badddba1b941d0cf281aed9d1b42cca0e1ae
</commit_message>
<xml_diff>
--- a/doc/GDRI-Indicatorlist.xlsx
+++ b/doc/GDRI-Indicatorlist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gla-my.sharepoint.com/personal/emilie_cremin_glasgow_ac_uk/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{0BE50E45-1472-E740-AAC2-E44E4C52637F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30BD5937-D1AF-3044-B6D5-221184514E66}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{0BE50E45-1472-E740-AAC2-E44E4C52637F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{937598F1-AA76-3343-BBF2-F76F4F0E43E5}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{CE13D24A-7942-F949-9FBF-79BC0511A8A2}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$151</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$U$152</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1291" uniqueCount="798">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1295" uniqueCount="800">
   <si>
     <t>code GDRI</t>
   </si>
@@ -1425,9 +1425,6 @@
     <t>ER_RES2</t>
   </si>
   <si>
-    <t>% of forest / mangrove area restored</t>
-  </si>
-  <si>
     <t>Forest Cover Change</t>
   </si>
   <si>
@@ -1779,9 +1776,6 @@
   </si>
   <si>
     <t>Yes</t>
-  </si>
-  <si>
-    <t>15.1.1 Forest area as a proportion of total land area/ Percentage of deforested area (%)  Percentage of net increase/decrease in mangrove area (%)</t>
   </si>
   <si>
     <t>2000 to 2020</t>
@@ -2879,6 +2873,18 @@
   </si>
   <si>
     <t>http://iridl.ldeo.columbia.edu/maproom/Global/Drought/Global/CPC_GOB/Analysis.html</t>
+  </si>
+  <si>
+    <t>ES_DES_1511</t>
+  </si>
+  <si>
+    <t>15.1.1 Forest area as a proportion of total land area</t>
+  </si>
+  <si>
+    <t>Percentage of deforested area (%)  or decrease in mangrove area (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% of forest / mangrove area restored (Forest gain) </t>
   </si>
 </sst>
 </file>
@@ -3412,7 +3418,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576F2231-92F9-2048-8A13-39208F3A7342}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:U154"/>
+  <dimension ref="A1:U155"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.6640625" style="5" customWidth="1"/>
@@ -3536,7 +3542,7 @@
       <c r="T2" s="4"/>
       <c r="U2" s="4"/>
     </row>
-    <row r="3" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" ht="82" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>28</v>
       </c>
@@ -3893,7 +3899,7 @@
       <c r="T11" s="4"/>
       <c r="U11" s="4"/>
     </row>
-    <row r="12" spans="1:21" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" ht="72" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>90</v>
       </c>
@@ -4303,7 +4309,7 @@
       <c r="T22" s="4"/>
       <c r="U22" s="4"/>
     </row>
-    <row r="23" spans="1:21" ht="82" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" ht="82" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>147</v>
       </c>
@@ -4580,7 +4586,7 @@
       <c r="T29" s="4"/>
       <c r="U29" s="4"/>
     </row>
-    <row r="30" spans="1:21" ht="204" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>189</v>
       </c>
@@ -4627,7 +4633,7 @@
       <c r="T30" s="4"/>
       <c r="U30" s="4"/>
     </row>
-    <row r="31" spans="1:21" ht="93" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:21" ht="93" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>197</v>
       </c>
@@ -5077,7 +5083,7 @@
       <c r="T42" s="4"/>
       <c r="U42" s="4"/>
     </row>
-    <row r="43" spans="1:21" ht="153" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>245</v>
       </c>
@@ -5122,7 +5128,7 @@
       <c r="T43" s="4"/>
       <c r="U43" s="4"/>
     </row>
-    <row r="44" spans="1:21" ht="187" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>251</v>
       </c>
@@ -5278,7 +5284,7 @@
       <c r="T47" s="4"/>
       <c r="U47" s="4"/>
     </row>
-    <row r="48" spans="1:21" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:21" ht="72" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>275</v>
       </c>
@@ -5320,7 +5326,7 @@
       <c r="T48" s="4"/>
       <c r="U48" s="4"/>
     </row>
-    <row r="49" spans="1:21" ht="162" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:21" ht="162" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>283</v>
       </c>
@@ -5362,7 +5368,7 @@
       <c r="T49" s="4"/>
       <c r="U49" s="4"/>
     </row>
-    <row r="50" spans="1:21" ht="83" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:21" ht="83" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>289</v>
       </c>
@@ -5402,7 +5408,7 @@
       <c r="T50" s="4"/>
       <c r="U50" s="4"/>
     </row>
-    <row r="51" spans="1:21" ht="60" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:21" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>295</v>
       </c>
@@ -5435,7 +5441,7 @@
       </c>
       <c r="U51" s="4"/>
     </row>
-    <row r="52" spans="1:21" ht="116" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:21" ht="116" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>298</v>
       </c>
@@ -5587,7 +5593,7 @@
       <c r="T55" s="4"/>
       <c r="U55" s="4"/>
     </row>
-    <row r="56" spans="1:21" ht="56" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:21" ht="56" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>322</v>
       </c>
@@ -5766,7 +5772,7 @@
       </c>
       <c r="U60" s="4"/>
     </row>
-    <row r="61" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:21" ht="68" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>347</v>
       </c>
@@ -5803,7 +5809,7 @@
       <c r="T61" s="4"/>
       <c r="U61" s="4"/>
     </row>
-    <row r="62" spans="1:21" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" ht="409.5" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>350</v>
       </c>
@@ -5840,7 +5846,7 @@
       <c r="T62" s="4"/>
       <c r="U62" s="4"/>
     </row>
-    <row r="63" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:21" ht="51" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>356</v>
       </c>
@@ -5871,7 +5877,7 @@
       <c r="T63" s="4"/>
       <c r="U63" s="4"/>
     </row>
-    <row r="64" spans="1:21" ht="66" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:21" ht="66" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>358</v>
       </c>
@@ -5952,7 +5958,7 @@
       <c r="T65" s="4"/>
       <c r="U65" s="4"/>
     </row>
-    <row r="66" spans="1:21" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:21" ht="119" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>371</v>
       </c>
@@ -6040,7 +6046,7 @@
       <c r="T67" s="4"/>
       <c r="U67" s="4"/>
     </row>
-    <row r="68" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:21" ht="136" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>384</v>
       </c>
@@ -6124,7 +6130,7 @@
       <c r="T69" s="4"/>
       <c r="U69" s="4"/>
     </row>
-    <row r="70" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:21" ht="34" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>393</v>
       </c>
@@ -6157,7 +6163,7 @@
       <c r="T70" s="4"/>
       <c r="U70" s="4"/>
     </row>
-    <row r="71" spans="1:21" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:21" ht="85" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>398</v>
       </c>
@@ -6171,39 +6177,39 @@
         <v>360</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>399</v>
+        <v>799</v>
       </c>
       <c r="J71" s="8"/>
       <c r="K71" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L71" s="4" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="M71" s="4" t="s">
         <v>397</v>
       </c>
       <c r="N71" s="4"/>
       <c r="O71" s="6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="P71" s="6"/>
       <c r="Q71" s="4"/>
       <c r="R71" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="S71" s="4" t="s">
         <v>402</v>
-      </c>
-      <c r="S71" s="4" t="s">
-        <v>403</v>
       </c>
       <c r="T71" s="4"/>
       <c r="U71" s="4"/>
     </row>
-    <row r="72" spans="1:21" ht="73" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:21" ht="73" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="B72" s="9" t="s">
         <v>404</v>
-      </c>
-      <c r="B72" s="9" t="s">
-        <v>405</v>
       </c>
       <c r="C72" s="9"/>
       <c r="D72" s="9" t="s">
@@ -6215,10 +6221,10 @@
         <v>332</v>
       </c>
       <c r="H72" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="I72" s="8" t="s">
         <v>406</v>
-      </c>
-      <c r="I72" s="8" t="s">
-        <v>407</v>
       </c>
       <c r="J72" s="8"/>
       <c r="K72" s="4" t="s">
@@ -6235,12 +6241,12 @@
       <c r="T72" s="4"/>
       <c r="U72" s="4"/>
     </row>
-    <row r="73" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:21" ht="170" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="B73" s="9" t="s">
         <v>408</v>
-      </c>
-      <c r="B73" s="9" t="s">
-        <v>409</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="9" t="s">
@@ -6255,47 +6261,47 @@
         <v>124</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="J73" s="8"/>
       <c r="K73" s="4"/>
       <c r="L73" s="4"/>
       <c r="M73" s="6" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="N73" s="6"/>
       <c r="O73" s="6" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="P73" s="6"/>
       <c r="Q73" s="4"/>
       <c r="R73" s="8" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="S73" s="4"/>
       <c r="T73" s="4"/>
       <c r="U73" s="4" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="74" spans="1:21" ht="204" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B74" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="B74" s="2" t="s">
+      <c r="D74" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="D74" s="2" t="s">
+      <c r="G74" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="G74" s="3" t="s">
+      <c r="H74" s="10" t="s">
         <v>418</v>
       </c>
-      <c r="H74" s="10" t="s">
+      <c r="I74" s="10" t="s">
         <v>419</v>
-      </c>
-      <c r="I74" s="10" t="s">
-        <v>420</v>
       </c>
       <c r="J74" s="10"/>
       <c r="K74" s="4"/>
@@ -6306,7 +6312,7 @@
       <c r="P74" s="4"/>
       <c r="Q74" s="4"/>
       <c r="R74" s="4" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
       <c r="S74" s="4"/>
       <c r="T74" s="4"/>
@@ -6314,120 +6320,120 @@
     </row>
     <row r="75" spans="1:21" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="B75" s="2" t="s">
         <v>422</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>423</v>
       </c>
       <c r="D75" s="2">
         <v>3</v>
       </c>
       <c r="G75" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="H75" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="H75" s="4" t="s">
-        <v>419</v>
-      </c>
       <c r="I75" s="8" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="J75" s="8"/>
       <c r="K75" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L75" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="M75" s="6" t="s">
         <v>425</v>
-      </c>
-      <c r="M75" s="6" t="s">
-        <v>426</v>
       </c>
       <c r="N75" s="6"/>
       <c r="O75" s="6" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="P75" s="6"/>
       <c r="Q75" s="6" t="s">
+        <v>427</v>
+      </c>
+      <c r="R75" s="4" t="s">
         <v>428</v>
       </c>
-      <c r="R75" s="4" t="s">
+      <c r="S75" s="4" t="s">
         <v>429</v>
-      </c>
-      <c r="S75" s="4" t="s">
-        <v>430</v>
       </c>
       <c r="T75" s="4"/>
       <c r="U75" s="4"/>
     </row>
     <row r="76" spans="1:21" ht="85" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
       <c r="D76" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G76" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="H76" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="H76" s="4" t="s">
-        <v>419</v>
-      </c>
       <c r="I76" s="8" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="J76" s="8"/>
       <c r="K76" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L76" s="4" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="M76" s="4"/>
       <c r="N76" s="4"/>
       <c r="O76" s="6" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="P76" s="6"/>
       <c r="Q76" s="4"/>
       <c r="R76" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="S76" s="4" t="s">
         <v>435</v>
-      </c>
-      <c r="S76" s="4" t="s">
-        <v>436</v>
       </c>
       <c r="T76" s="4"/>
       <c r="U76" s="4"/>
     </row>
     <row r="77" spans="1:21" ht="128" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
+        <v>436</v>
+      </c>
+      <c r="B77" s="2" t="s">
         <v>437</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>438</v>
       </c>
       <c r="D77" s="2">
         <v>3</v>
       </c>
       <c r="G77" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H77" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="I77" s="10" t="s">
         <v>439</v>
-      </c>
-      <c r="I77" s="10" t="s">
-        <v>440</v>
       </c>
       <c r="J77" s="10"/>
       <c r="K77" s="4"/>
       <c r="L77" s="4"/>
       <c r="M77" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="N77" s="4"/>
       <c r="O77" s="4"/>
       <c r="P77" s="4"/>
       <c r="Q77" s="4"/>
       <c r="R77" s="4" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="S77" s="4"/>
       <c r="T77" s="4"/>
@@ -6435,22 +6441,22 @@
     </row>
     <row r="78" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B78" s="2" t="s">
         <v>443</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>444</v>
       </c>
       <c r="D78" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G78" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="J78" s="10"/>
       <c r="K78" s="4"/>
@@ -6461,7 +6467,7 @@
       <c r="P78" s="4"/>
       <c r="Q78" s="4"/>
       <c r="R78" s="4" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="S78" s="4"/>
       <c r="T78" s="4"/>
@@ -6469,10 +6475,10 @@
     </row>
     <row r="79" spans="1:21" ht="61" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
+        <v>446</v>
+      </c>
+      <c r="B79" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>448</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>64</v>
@@ -6481,13 +6487,13 @@
         <v>3</v>
       </c>
       <c r="G79" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I79" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="J79" s="4"/>
       <c r="K79" s="4"/>
@@ -6498,7 +6504,7 @@
       <c r="P79" s="4"/>
       <c r="Q79" s="4"/>
       <c r="R79" s="4" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="S79" s="4"/>
       <c r="T79" s="4"/>
@@ -6506,19 +6512,19 @@
     </row>
     <row r="80" spans="1:21" ht="136" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D80" s="2">
         <v>3</v>
       </c>
       <c r="G80" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H80" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I80" s="8" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="J80" s="8"/>
       <c r="K80" s="4" t="s">
@@ -6526,46 +6532,46 @@
       </c>
       <c r="L80" s="4"/>
       <c r="M80" s="6" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="N80" s="6"/>
       <c r="O80" s="6" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="P80" s="6"/>
       <c r="Q80" s="6"/>
       <c r="R80" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="S80" s="4" t="s">
         <v>455</v>
-      </c>
-      <c r="S80" s="4" t="s">
-        <v>456</v>
       </c>
       <c r="T80" s="4"/>
       <c r="U80" s="4"/>
     </row>
     <row r="81" spans="1:21" ht="136" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="G81" s="3"/>
       <c r="H81" s="4"/>
       <c r="I81" s="8" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="J81" s="8"/>
       <c r="K81" s="4"/>
       <c r="L81" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="M81" s="6" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="N81" s="6"/>
       <c r="O81" s="6"/>
       <c r="P81" s="6"/>
       <c r="Q81" s="6"/>
       <c r="R81" s="4" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="S81" s="4"/>
       <c r="T81" s="4"/>
@@ -6573,51 +6579,51 @@
     </row>
     <row r="82" spans="1:21" ht="118" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D82" s="2">
         <v>3</v>
       </c>
       <c r="G82" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I82" s="4" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="J82" s="4"/>
       <c r="K82" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L82" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="M82" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="N82" s="4"/>
       <c r="O82" s="6" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="P82" s="6"/>
       <c r="Q82" s="4"/>
       <c r="R82" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="S82" s="4" t="s">
         <v>465</v>
-      </c>
-      <c r="S82" s="4" t="s">
-        <v>466</v>
       </c>
       <c r="T82" s="4"/>
       <c r="U82" s="4"/>
     </row>
-    <row r="83" spans="1:21" ht="117" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:21" ht="117" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
+        <v>466</v>
+      </c>
+      <c r="B83" s="9" t="s">
         <v>467</v>
-      </c>
-      <c r="B83" s="9" t="s">
-        <v>468</v>
       </c>
       <c r="C83" s="9"/>
       <c r="D83" s="9">
@@ -6628,47 +6634,47 @@
         <v>92</v>
       </c>
       <c r="G83" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H83" s="4" t="s">
         <v>124</v>
       </c>
       <c r="I83" s="8" t="s">
+        <v>468</v>
+      </c>
+      <c r="J83" s="8" t="s">
         <v>469</v>
-      </c>
-      <c r="J83" s="8" t="s">
-        <v>470</v>
       </c>
       <c r="K83" s="4"/>
       <c r="L83" s="4"/>
       <c r="M83" s="6" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="N83" s="6"/>
       <c r="O83" s="4"/>
       <c r="P83" s="4"/>
       <c r="Q83" s="4"/>
       <c r="R83" s="8" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="S83" s="4"/>
       <c r="T83" s="4" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="U83" s="4"/>
     </row>
     <row r="84" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D84" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G84" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H84" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I84" s="8" t="s">
         <v>344</v>
@@ -6678,41 +6684,41 @@
         <v>25</v>
       </c>
       <c r="L84" s="16" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="M84" s="4"/>
       <c r="N84" s="4"/>
       <c r="O84" s="6" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="P84" s="6"/>
       <c r="Q84" s="4"/>
       <c r="R84" s="4" t="s">
+        <v>474</v>
+      </c>
+      <c r="S84" s="4" t="s">
         <v>475</v>
       </c>
-      <c r="S84" s="4" t="s">
+      <c r="T84" s="8" t="s">
         <v>476</v>
-      </c>
-      <c r="T84" s="8" t="s">
-        <v>477</v>
       </c>
       <c r="U84" s="4"/>
     </row>
     <row r="85" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="D85" s="2">
         <v>3</v>
       </c>
       <c r="G85" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H85" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="I85" s="8" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="J85" s="8"/>
       <c r="K85" s="4" t="s">
@@ -6722,282 +6728,275 @@
       <c r="M85" s="4"/>
       <c r="N85" s="4"/>
       <c r="O85" s="6" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="P85" s="6"/>
       <c r="Q85" s="4"/>
       <c r="R85" s="4" t="s">
+        <v>480</v>
+      </c>
+      <c r="S85" s="4" t="s">
         <v>481</v>
-      </c>
-      <c r="S85" s="4" t="s">
-        <v>482</v>
       </c>
       <c r="T85" s="8"/>
       <c r="U85" s="4"/>
     </row>
-    <row r="86" spans="1:21" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:21" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D86" s="2">
         <v>3</v>
       </c>
       <c r="F86" s="2" t="s">
+        <v>483</v>
+      </c>
+      <c r="G86" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="H86" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="G86" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="H86" s="4" t="s">
+      <c r="I86" s="8" t="s">
         <v>485</v>
-      </c>
-      <c r="I86" s="8" t="s">
-        <v>486</v>
       </c>
       <c r="J86" s="8"/>
       <c r="K86" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L86" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="M86" s="21" t="s">
         <v>487</v>
-      </c>
-      <c r="M86" s="21" t="s">
-        <v>488</v>
       </c>
       <c r="N86" s="21"/>
       <c r="O86" s="6" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="P86" s="6"/>
       <c r="Q86" s="4"/>
       <c r="R86" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="S86" s="8" t="s">
         <v>490</v>
       </c>
-      <c r="S86" s="8" t="s">
+      <c r="T86" s="8" t="s">
         <v>491</v>
       </c>
-      <c r="T86" s="8" t="s">
+      <c r="U86" s="4"/>
+    </row>
+    <row r="87" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
+        <v>796</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="G87" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>797</v>
+      </c>
+      <c r="J87" s="8"/>
+      <c r="K87" s="4"/>
+      <c r="L87" s="4"/>
+      <c r="M87" s="21"/>
+      <c r="N87" s="21"/>
+      <c r="O87" s="6"/>
+      <c r="P87" s="6"/>
+      <c r="Q87" s="4"/>
+      <c r="R87" s="4"/>
+      <c r="S87" s="8"/>
+      <c r="T87" s="8"/>
+      <c r="U87" s="4"/>
+    </row>
+    <row r="88" spans="1:21" ht="372" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="U86" s="4"/>
-    </row>
-    <row r="87" spans="1:21" ht="372" x14ac:dyDescent="0.2">
-      <c r="A87" s="1" t="s">
-        <v>493</v>
-      </c>
-      <c r="B87" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>494</v>
       </c>
-      <c r="D87" s="2" t="s">
-        <v>495</v>
-      </c>
-      <c r="F87" s="2" t="s">
-        <v>484</v>
-      </c>
-      <c r="G87" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="H87" s="4" t="s">
-        <v>439</v>
-      </c>
-      <c r="I87" s="8" t="s">
-        <v>496</v>
-      </c>
-      <c r="J87" s="8"/>
-      <c r="K87" s="4" t="s">
-        <v>497</v>
-      </c>
-      <c r="L87" s="4" t="s">
-        <v>498</v>
-      </c>
-      <c r="M87" s="21" t="s">
-        <v>499</v>
-      </c>
-      <c r="N87" s="21"/>
-      <c r="O87" s="8" t="s">
-        <v>500</v>
-      </c>
-      <c r="P87" s="8"/>
-      <c r="Q87" s="4"/>
-      <c r="R87" s="8" t="s">
-        <v>501</v>
-      </c>
-      <c r="S87" s="8" t="s">
-        <v>502</v>
-      </c>
-      <c r="T87" s="8" t="s">
-        <v>503</v>
-      </c>
-      <c r="U87" s="4"/>
-    </row>
-    <row r="88" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="1" t="s">
-        <v>504</v>
-      </c>
-      <c r="D88" s="2">
-        <v>3</v>
+      <c r="F88" s="2" t="s">
+        <v>483</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H88" s="4" t="s">
-        <v>505</v>
+        <v>438</v>
       </c>
       <c r="I88" s="8" t="s">
-        <v>506</v>
+        <v>798</v>
       </c>
       <c r="J88" s="8"/>
       <c r="K88" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L88" s="4"/>
-      <c r="M88" s="6" t="s">
-        <v>454</v>
-      </c>
-      <c r="N88" s="6"/>
-      <c r="O88" s="4"/>
-      <c r="P88" s="4"/>
+        <v>495</v>
+      </c>
+      <c r="L88" s="4" t="s">
+        <v>496</v>
+      </c>
+      <c r="M88" s="21" t="s">
+        <v>497</v>
+      </c>
+      <c r="N88" s="21"/>
+      <c r="O88" s="8" t="s">
+        <v>498</v>
+      </c>
+      <c r="P88" s="8"/>
       <c r="Q88" s="4"/>
-      <c r="R88" s="4"/>
-      <c r="S88" s="4"/>
-      <c r="T88" s="4"/>
+      <c r="R88" s="8" t="s">
+        <v>499</v>
+      </c>
+      <c r="S88" s="8" t="s">
+        <v>500</v>
+      </c>
+      <c r="T88" s="8" t="s">
+        <v>501</v>
+      </c>
       <c r="U88" s="4"/>
     </row>
-    <row r="89" spans="1:21" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="D89" s="2">
         <v>3</v>
       </c>
       <c r="G89" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>505</v>
-      </c>
-      <c r="I89" s="4" t="s">
-        <v>508</v>
-      </c>
-      <c r="J89" s="4"/>
+        <v>503</v>
+      </c>
+      <c r="I89" s="8" t="s">
+        <v>504</v>
+      </c>
+      <c r="J89" s="8"/>
       <c r="K89" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L89" s="4"/>
-      <c r="M89" s="4" t="s">
-        <v>509</v>
-      </c>
-      <c r="N89" s="4"/>
-      <c r="O89" s="4" t="s">
-        <v>510</v>
-      </c>
+      <c r="M89" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="N89" s="6"/>
+      <c r="O89" s="4"/>
       <c r="P89" s="4"/>
       <c r="Q89" s="4"/>
-      <c r="R89" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="S89" s="8" t="s">
-        <v>512</v>
-      </c>
-      <c r="T89" s="8" t="s">
-        <v>513</v>
-      </c>
+      <c r="R89" s="4"/>
+      <c r="S89" s="4"/>
+      <c r="T89" s="4"/>
       <c r="U89" s="4"/>
     </row>
-    <row r="90" spans="1:21" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:21" ht="409.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
-        <v>514</v>
+        <v>505</v>
       </c>
       <c r="D90" s="2">
         <v>3</v>
       </c>
-      <c r="F90" s="2" t="s">
-        <v>149</v>
-      </c>
       <c r="G90" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="I90" s="4" t="s">
-        <v>515</v>
+        <v>506</v>
       </c>
       <c r="J90" s="4"/>
       <c r="K90" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L90" s="4"/>
-      <c r="M90" s="6" t="s">
-        <v>516</v>
-      </c>
-      <c r="N90" s="6"/>
-      <c r="O90" s="8" t="s">
-        <v>517</v>
-      </c>
-      <c r="P90" s="8"/>
+      <c r="M90" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="N90" s="4"/>
+      <c r="O90" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="P90" s="4"/>
       <c r="Q90" s="4"/>
       <c r="R90" s="4" t="s">
-        <v>518</v>
-      </c>
-      <c r="S90" s="4" t="s">
-        <v>519</v>
+        <v>509</v>
+      </c>
+      <c r="S90" s="8" t="s">
+        <v>510</v>
       </c>
       <c r="T90" s="8" t="s">
-        <v>520</v>
+        <v>511</v>
       </c>
       <c r="U90" s="4"/>
     </row>
-    <row r="91" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:21" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
-        <v>521</v>
+        <v>512</v>
       </c>
       <c r="D91" s="2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>149</v>
       </c>
       <c r="G91" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="I91" s="4" t="s">
-        <v>522</v>
+        <v>513</v>
       </c>
       <c r="J91" s="4"/>
       <c r="K91" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L91" s="4"/>
-      <c r="M91" s="4"/>
-      <c r="N91" s="4"/>
-      <c r="O91" s="4"/>
-      <c r="P91" s="4"/>
+      <c r="M91" s="6" t="s">
+        <v>514</v>
+      </c>
+      <c r="N91" s="6"/>
+      <c r="O91" s="8" t="s">
+        <v>515</v>
+      </c>
+      <c r="P91" s="8"/>
       <c r="Q91" s="4"/>
       <c r="R91" s="4" t="s">
-        <v>523</v>
-      </c>
-      <c r="S91" s="4"/>
-      <c r="T91" s="4"/>
+        <v>516</v>
+      </c>
+      <c r="S91" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="T91" s="8" t="s">
+        <v>518</v>
+      </c>
       <c r="U91" s="4"/>
     </row>
-    <row r="92" spans="1:21" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
-        <v>524</v>
+        <v>519</v>
       </c>
       <c r="D92" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G92" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H92" s="4" t="s">
-        <v>525</v>
-      </c>
-      <c r="I92" s="8" t="s">
-        <v>526</v>
-      </c>
-      <c r="J92" s="8"/>
+        <v>503</v>
+      </c>
+      <c r="I92" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="J92" s="4"/>
       <c r="K92" s="4" t="s">
         <v>25</v>
       </c>
@@ -7008,33 +7007,29 @@
       <c r="P92" s="4"/>
       <c r="Q92" s="4"/>
       <c r="R92" s="4" t="s">
-        <v>527</v>
-      </c>
-      <c r="S92" s="4" t="s">
-        <v>528</v>
-      </c>
-      <c r="T92" s="8" t="s">
-        <v>529</v>
-      </c>
+        <v>521</v>
+      </c>
+      <c r="S92" s="4"/>
+      <c r="T92" s="4"/>
       <c r="U92" s="4"/>
     </row>
-    <row r="93" spans="1:21" ht="165" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:21" ht="409.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
-        <v>530</v>
+        <v>522</v>
       </c>
       <c r="D93" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G93" s="3" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="I93" s="4" t="s">
-        <v>531</v>
-      </c>
-      <c r="J93" s="4"/>
+        <v>523</v>
+      </c>
+      <c r="I93" s="8" t="s">
+        <v>524</v>
+      </c>
+      <c r="J93" s="8"/>
       <c r="K93" s="4" t="s">
         <v>25</v>
       </c>
@@ -7044,32 +7039,37 @@
       <c r="O93" s="4"/>
       <c r="P93" s="4"/>
       <c r="Q93" s="4"/>
-      <c r="R93" s="4"/>
-      <c r="S93" s="4"/>
-      <c r="T93" s="4"/>
+      <c r="R93" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="S93" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="T93" s="8" t="s">
+        <v>527</v>
+      </c>
       <c r="U93" s="4"/>
     </row>
-    <row r="94" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:21" ht="165" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
-        <v>532</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>533</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>39</v>
+        <v>528</v>
+      </c>
+      <c r="D94" s="2">
+        <v>3</v>
       </c>
       <c r="G94" s="3" t="s">
-        <v>534</v>
+        <v>417</v>
       </c>
       <c r="H94" s="4" t="s">
-        <v>40</v>
+        <v>333</v>
       </c>
       <c r="I94" s="4" t="s">
-        <v>535</v>
+        <v>529</v>
       </c>
       <c r="J94" s="4"/>
-      <c r="K94" s="4"/>
+      <c r="K94" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="L94" s="4"/>
       <c r="M94" s="4"/>
       <c r="N94" s="4"/>
@@ -7081,55 +7081,44 @@
       <c r="T94" s="4"/>
       <c r="U94" s="4"/>
     </row>
-    <row r="95" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
-        <v>536</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>537</v>
+        <v>530</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="D95" s="2">
-        <v>3</v>
+        <v>531</v>
+      </c>
+      <c r="D95" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="G95" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H95" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="I95" s="10" t="s">
-        <v>539</v>
-      </c>
-      <c r="J95" s="10"/>
+        <v>532</v>
+      </c>
+      <c r="H95" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I95" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="J95" s="4"/>
       <c r="K95" s="4"/>
       <c r="L95" s="4"/>
-      <c r="M95" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="N95" s="6"/>
+      <c r="M95" s="4"/>
+      <c r="N95" s="4"/>
       <c r="O95" s="4"/>
       <c r="P95" s="4"/>
       <c r="Q95" s="4"/>
-      <c r="R95" s="8" t="s">
-        <v>541</v>
-      </c>
-      <c r="S95" s="8" t="s">
-        <v>542</v>
-      </c>
-      <c r="T95" s="4" t="s">
-        <v>543</v>
-      </c>
+      <c r="R95" s="4"/>
+      <c r="S95" s="4"/>
+      <c r="T95" s="4"/>
       <c r="U95" s="4"/>
     </row>
-    <row r="96" spans="1:21" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
-        <v>544</v>
+        <v>534</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>64</v>
@@ -7138,162 +7127,174 @@
         <v>3</v>
       </c>
       <c r="G96" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H96" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I96" s="10" t="s">
-        <v>546</v>
+        <v>537</v>
       </c>
       <c r="J96" s="10"/>
       <c r="K96" s="4"/>
       <c r="L96" s="4"/>
-      <c r="M96" s="4"/>
-      <c r="N96" s="4"/>
+      <c r="M96" s="6" t="s">
+        <v>538</v>
+      </c>
+      <c r="N96" s="6"/>
       <c r="O96" s="4"/>
       <c r="P96" s="4"/>
       <c r="Q96" s="4"/>
-      <c r="R96" s="4"/>
+      <c r="R96" s="8" t="s">
+        <v>539</v>
+      </c>
       <c r="S96" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="T96" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="U96" s="4"/>
+    </row>
+    <row r="97" spans="1:21" ht="64" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
         <v>542</v>
       </c>
-      <c r="T96" s="4" t="s">
+      <c r="B97" s="2" t="s">
         <v>543</v>
       </c>
-      <c r="U96" s="4"/>
-    </row>
-    <row r="97" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="1" t="s">
-        <v>547</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>548</v>
+      <c r="C97" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="D97" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G97" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H97" s="10" t="s">
         <v>56</v>
       </c>
       <c r="I97" s="10" t="s">
-        <v>549</v>
+        <v>544</v>
       </c>
       <c r="J97" s="10"/>
       <c r="K97" s="4"/>
       <c r="L97" s="4"/>
-      <c r="M97" s="6" t="s">
-        <v>550</v>
-      </c>
-      <c r="N97" s="6"/>
+      <c r="M97" s="4"/>
+      <c r="N97" s="4"/>
       <c r="O97" s="4"/>
       <c r="P97" s="4"/>
       <c r="Q97" s="4"/>
-      <c r="R97" s="8" t="s">
-        <v>551</v>
-      </c>
-      <c r="S97" s="4" t="s">
-        <v>552</v>
-      </c>
-      <c r="T97" s="4"/>
+      <c r="R97" s="4"/>
+      <c r="S97" s="8" t="s">
+        <v>540</v>
+      </c>
+      <c r="T97" s="4" t="s">
+        <v>541</v>
+      </c>
       <c r="U97" s="4"/>
     </row>
-    <row r="98" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
-        <v>553</v>
+        <v>545</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>546</v>
       </c>
       <c r="D98" s="2">
         <v>2</v>
       </c>
       <c r="G98" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H98" s="4" t="s">
-        <v>554</v>
-      </c>
-      <c r="I98" s="4" t="s">
-        <v>555</v>
-      </c>
-      <c r="J98" s="4"/>
-      <c r="K98" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L98" s="4" t="s">
-        <v>556</v>
-      </c>
-      <c r="M98" s="4"/>
-      <c r="N98" s="4"/>
+        <v>536</v>
+      </c>
+      <c r="H98" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="I98" s="10" t="s">
+        <v>547</v>
+      </c>
+      <c r="J98" s="10"/>
+      <c r="K98" s="4"/>
+      <c r="L98" s="4"/>
+      <c r="M98" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="N98" s="6"/>
       <c r="O98" s="4"/>
       <c r="P98" s="4"/>
       <c r="Q98" s="4"/>
-      <c r="R98" s="4"/>
-      <c r="S98" s="4"/>
-      <c r="T98" s="8" t="s">
-        <v>557</v>
-      </c>
+      <c r="R98" s="8" t="s">
+        <v>549</v>
+      </c>
+      <c r="S98" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="T98" s="4"/>
       <c r="U98" s="4"/>
     </row>
-    <row r="99" spans="1:21" ht="53" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="D99" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G99" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H99" s="4" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="I99" s="4" t="s">
-        <v>559</v>
+        <v>553</v>
       </c>
       <c r="J99" s="4"/>
       <c r="K99" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L99" s="4" t="s">
-        <v>556</v>
-      </c>
-      <c r="M99" s="6" t="s">
-        <v>560</v>
-      </c>
-      <c r="N99" s="6"/>
+        <v>554</v>
+      </c>
+      <c r="M99" s="4"/>
+      <c r="N99" s="4"/>
       <c r="O99" s="4"/>
       <c r="P99" s="4"/>
       <c r="Q99" s="4"/>
       <c r="R99" s="4"/>
       <c r="S99" s="4"/>
-      <c r="T99" s="4"/>
+      <c r="T99" s="8" t="s">
+        <v>555</v>
+      </c>
       <c r="U99" s="4"/>
     </row>
-    <row r="100" spans="1:21" ht="56" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:21" ht="53" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
-        <v>561</v>
-      </c>
-      <c r="D100" s="2" t="s">
-        <v>82</v>
+        <v>556</v>
+      </c>
+      <c r="D100" s="2">
+        <v>3</v>
       </c>
       <c r="G100" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H100" s="4" t="s">
-        <v>554</v>
-      </c>
-      <c r="I100" s="8" t="s">
-        <v>562</v>
-      </c>
-      <c r="J100" s="8"/>
+        <v>552</v>
+      </c>
+      <c r="I100" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="J100" s="4"/>
       <c r="K100" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L100" s="4"/>
-      <c r="M100" s="4"/>
-      <c r="N100" s="4"/>
+      <c r="L100" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="M100" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="N100" s="6"/>
       <c r="O100" s="4"/>
       <c r="P100" s="4"/>
       <c r="Q100" s="4"/>
@@ -7302,63 +7303,58 @@
       <c r="T100" s="4"/>
       <c r="U100" s="4"/>
     </row>
-    <row r="101" spans="1:21" ht="68" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:21" ht="56" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
-        <v>563</v>
-      </c>
-      <c r="B101" s="2" t="s">
-        <v>564</v>
-      </c>
-      <c r="D101" s="2">
-        <v>3</v>
+        <v>559</v>
+      </c>
+      <c r="D101" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H101" s="10" t="s">
-        <v>565</v>
-      </c>
-      <c r="I101" s="10" t="s">
-        <v>566</v>
-      </c>
-      <c r="J101" s="10"/>
-      <c r="K101" s="4"/>
+        <v>536</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="I101" s="8" t="s">
+        <v>560</v>
+      </c>
+      <c r="J101" s="8"/>
+      <c r="K101" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="L101" s="4"/>
       <c r="M101" s="4"/>
       <c r="N101" s="4"/>
       <c r="O101" s="4"/>
       <c r="P101" s="4"/>
       <c r="Q101" s="4"/>
-      <c r="R101" s="4" t="s">
-        <v>567</v>
-      </c>
+      <c r="R101" s="4"/>
       <c r="S101" s="4"/>
       <c r="T101" s="4"/>
       <c r="U101" s="4"/>
     </row>
-    <row r="102" spans="1:21" ht="238" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:21" ht="68" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
-        <v>568</v>
+        <v>561</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>569</v>
+        <v>562</v>
       </c>
       <c r="D102" s="2">
         <v>3</v>
       </c>
       <c r="G102" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H102" s="4" t="s">
-        <v>565</v>
-      </c>
-      <c r="I102" s="4" t="s">
-        <v>570</v>
-      </c>
-      <c r="J102" s="4"/>
-      <c r="K102" s="4" t="s">
-        <v>25</v>
-      </c>
+        <v>536</v>
+      </c>
+      <c r="H102" s="10" t="s">
+        <v>563</v>
+      </c>
+      <c r="I102" s="10" t="s">
+        <v>564</v>
+      </c>
+      <c r="J102" s="10"/>
+      <c r="K102" s="4"/>
       <c r="L102" s="4"/>
       <c r="M102" s="4"/>
       <c r="N102" s="4"/>
@@ -7366,32 +7362,30 @@
       <c r="P102" s="4"/>
       <c r="Q102" s="4"/>
       <c r="R102" s="4" t="s">
-        <v>571</v>
-      </c>
-      <c r="S102" s="8" t="s">
-        <v>572</v>
-      </c>
+        <v>565</v>
+      </c>
+      <c r="S102" s="4"/>
       <c r="T102" s="4"/>
       <c r="U102" s="4"/>
     </row>
-    <row r="103" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:21" ht="238" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
-        <v>573</v>
+        <v>566</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>574</v>
+        <v>567</v>
       </c>
       <c r="D103" s="2">
         <v>3</v>
       </c>
       <c r="G103" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H103" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I103" s="4" t="s">
-        <v>575</v>
+        <v>568</v>
       </c>
       <c r="J103" s="4"/>
       <c r="K103" s="4" t="s">
@@ -7403,29 +7397,33 @@
       <c r="O103" s="4"/>
       <c r="P103" s="4"/>
       <c r="Q103" s="4"/>
-      <c r="R103" s="4"/>
-      <c r="S103" s="4"/>
+      <c r="R103" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="S103" s="8" t="s">
+        <v>570</v>
+      </c>
       <c r="T103" s="4"/>
       <c r="U103" s="4"/>
     </row>
-    <row r="104" spans="1:21" ht="75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
-        <v>576</v>
+        <v>571</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>82</v>
+        <v>572</v>
+      </c>
+      <c r="D104" s="2">
+        <v>3</v>
       </c>
       <c r="G104" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H104" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I104" s="4" t="s">
-        <v>578</v>
+        <v>573</v>
       </c>
       <c r="J104" s="4"/>
       <c r="K104" s="4" t="s">
@@ -7442,21 +7440,24 @@
       <c r="T104" s="4"/>
       <c r="U104" s="4"/>
     </row>
-    <row r="105" spans="1:21" ht="84" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:21" ht="75" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
-        <v>579</v>
+        <v>574</v>
+      </c>
+      <c r="B105" s="2" t="s">
+        <v>575</v>
       </c>
       <c r="D105" s="2" t="s">
         <v>82</v>
       </c>
       <c r="G105" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H105" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I105" s="4" t="s">
-        <v>580</v>
+        <v>576</v>
       </c>
       <c r="J105" s="4"/>
       <c r="K105" s="4" t="s">
@@ -7473,21 +7474,21 @@
       <c r="T105" s="4"/>
       <c r="U105" s="4"/>
     </row>
-    <row r="106" spans="1:21" ht="62" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:21" ht="84" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
-        <v>581</v>
+        <v>577</v>
       </c>
       <c r="D106" s="2" t="s">
         <v>82</v>
       </c>
       <c r="G106" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H106" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I106" s="4" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="J106" s="4"/>
       <c r="K106" s="4" t="s">
@@ -7504,24 +7505,21 @@
       <c r="T106" s="4"/>
       <c r="U106" s="4"/>
     </row>
-    <row r="107" spans="1:21" ht="108" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:21" ht="62" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
-        <v>583</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>584</v>
-      </c>
-      <c r="D107" s="2">
-        <v>3</v>
+        <v>579</v>
+      </c>
+      <c r="D107" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="G107" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H107" s="4" t="s">
-        <v>554</v>
+        <v>563</v>
       </c>
       <c r="I107" s="4" t="s">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="J107" s="4"/>
       <c r="K107" s="4" t="s">
@@ -7538,357 +7536,351 @@
       <c r="T107" s="4"/>
       <c r="U107" s="4"/>
     </row>
-    <row r="108" spans="1:21" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:21" ht="108" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>587</v>
-      </c>
-      <c r="D108" s="2" t="s">
-        <v>82</v>
+        <v>582</v>
+      </c>
+      <c r="D108" s="2">
+        <v>3</v>
       </c>
       <c r="G108" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H108" s="10" t="s">
-        <v>554</v>
-      </c>
-      <c r="I108" s="10" t="s">
-        <v>588</v>
-      </c>
-      <c r="J108" s="10"/>
-      <c r="K108" s="4"/>
+        <v>536</v>
+      </c>
+      <c r="H108" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="I108" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="J108" s="4"/>
+      <c r="K108" s="4" t="s">
+        <v>25</v>
+      </c>
       <c r="L108" s="4"/>
-      <c r="M108" s="6" t="s">
-        <v>589</v>
-      </c>
-      <c r="N108" s="6"/>
+      <c r="M108" s="4"/>
+      <c r="N108" s="4"/>
       <c r="O108" s="4"/>
       <c r="P108" s="4"/>
       <c r="Q108" s="4"/>
-      <c r="R108" s="8" t="s">
-        <v>590</v>
-      </c>
-      <c r="S108" s="4" t="s">
-        <v>591</v>
-      </c>
+      <c r="R108" s="4"/>
+      <c r="S108" s="4"/>
       <c r="T108" s="4"/>
       <c r="U108" s="4"/>
     </row>
-    <row r="109" spans="1:21" ht="131" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:21" ht="102" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
-        <v>592</v>
+        <v>584</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>593</v>
-      </c>
-      <c r="D109" s="2">
-        <v>3</v>
+        <v>585</v>
+      </c>
+      <c r="D109" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="G109" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H109" s="10" t="s">
-        <v>554</v>
+        <v>552</v>
       </c>
       <c r="I109" s="10" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="J109" s="10"/>
       <c r="K109" s="4"/>
       <c r="L109" s="4"/>
       <c r="M109" s="6" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="N109" s="6"/>
-      <c r="O109" s="6" t="s">
-        <v>595</v>
-      </c>
-      <c r="P109" s="6"/>
+      <c r="O109" s="4"/>
+      <c r="P109" s="4"/>
       <c r="Q109" s="4"/>
       <c r="R109" s="8" t="s">
-        <v>596</v>
-      </c>
-      <c r="S109" s="4"/>
+        <v>588</v>
+      </c>
+      <c r="S109" s="4" t="s">
+        <v>589</v>
+      </c>
       <c r="T109" s="4"/>
       <c r="U109" s="4"/>
     </row>
-    <row r="110" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:21" ht="131" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
-        <v>597</v>
+        <v>590</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="C110" s="2" t="s">
-        <v>599</v>
+        <v>591</v>
       </c>
       <c r="D110" s="2">
         <v>3</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H110" s="10" t="s">
-        <v>600</v>
+        <v>552</v>
       </c>
       <c r="I110" s="10" t="s">
-        <v>601</v>
+        <v>592</v>
       </c>
       <c r="J110" s="10"/>
       <c r="K110" s="4"/>
       <c r="L110" s="4"/>
-      <c r="M110" s="4"/>
-      <c r="N110" s="4"/>
-      <c r="O110" s="4"/>
-      <c r="P110" s="4"/>
+      <c r="M110" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="N110" s="6"/>
+      <c r="O110" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="P110" s="6"/>
       <c r="Q110" s="4"/>
-      <c r="R110" s="4" t="s">
-        <v>602</v>
-      </c>
-      <c r="S110" s="4" t="s">
-        <v>602</v>
-      </c>
+      <c r="R110" s="8" t="s">
+        <v>594</v>
+      </c>
+      <c r="S110" s="4"/>
       <c r="T110" s="4"/>
       <c r="U110" s="4"/>
     </row>
-    <row r="111" spans="1:21" ht="107" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
-        <v>603</v>
+        <v>595</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>604</v>
+        <v>596</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>597</v>
       </c>
       <c r="D111" s="2">
         <v>3</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H111" s="4" t="s">
-        <v>565</v>
-      </c>
-      <c r="I111" s="4" t="s">
-        <v>605</v>
-      </c>
-      <c r="J111" s="4"/>
-      <c r="K111" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L111" s="8" t="s">
-        <v>606</v>
-      </c>
-      <c r="M111" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="N111" s="8"/>
+        <v>536</v>
+      </c>
+      <c r="H111" s="10" t="s">
+        <v>598</v>
+      </c>
+      <c r="I111" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="J111" s="10"/>
+      <c r="K111" s="4"/>
+      <c r="L111" s="4"/>
+      <c r="M111" s="4"/>
+      <c r="N111" s="4"/>
       <c r="O111" s="4"/>
       <c r="P111" s="4"/>
       <c r="Q111" s="4"/>
       <c r="R111" s="4" t="s">
-        <v>571</v>
-      </c>
-      <c r="S111" s="8" t="s">
-        <v>572</v>
+        <v>600</v>
+      </c>
+      <c r="S111" s="4" t="s">
+        <v>600</v>
       </c>
       <c r="T111" s="4"/>
       <c r="U111" s="4"/>
     </row>
-    <row r="112" spans="1:21" ht="136" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:21" ht="107" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
-        <v>608</v>
+        <v>601</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>609</v>
+        <v>602</v>
       </c>
       <c r="D112" s="2">
         <v>3</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H112" s="10" t="s">
-        <v>565</v>
-      </c>
-      <c r="I112" s="10" t="s">
-        <v>610</v>
-      </c>
-      <c r="J112" s="10"/>
-      <c r="K112" s="4"/>
-      <c r="L112" s="4"/>
-      <c r="M112" s="4"/>
-      <c r="N112" s="4"/>
+        <v>536</v>
+      </c>
+      <c r="H112" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="I112" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="J112" s="4"/>
+      <c r="K112" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L112" s="8" t="s">
+        <v>604</v>
+      </c>
+      <c r="M112" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="N112" s="8"/>
       <c r="O112" s="4"/>
       <c r="P112" s="4"/>
       <c r="Q112" s="4"/>
-      <c r="R112" s="4"/>
-      <c r="S112" s="4"/>
+      <c r="R112" s="4" t="s">
+        <v>569</v>
+      </c>
+      <c r="S112" s="8" t="s">
+        <v>570</v>
+      </c>
       <c r="T112" s="4"/>
       <c r="U112" s="4"/>
     </row>
-    <row r="113" spans="1:21" ht="204" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:21" ht="136" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
-        <v>611</v>
-      </c>
-      <c r="D113" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="F113" s="2" t="s">
-        <v>92</v>
+        <v>606</v>
+      </c>
+      <c r="B113" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="D113" s="2">
+        <v>3</v>
       </c>
       <c r="G113" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H113" s="4" t="s">
-        <v>565</v>
-      </c>
-      <c r="I113" s="4" t="s">
-        <v>612</v>
-      </c>
-      <c r="J113" s="4"/>
-      <c r="K113" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L113" s="8"/>
-      <c r="M113" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="N113" s="8"/>
+        <v>536</v>
+      </c>
+      <c r="H113" s="10" t="s">
+        <v>563</v>
+      </c>
+      <c r="I113" s="10" t="s">
+        <v>608</v>
+      </c>
+      <c r="J113" s="10"/>
+      <c r="K113" s="4"/>
+      <c r="L113" s="4"/>
+      <c r="M113" s="4"/>
+      <c r="N113" s="4"/>
       <c r="O113" s="4"/>
       <c r="P113" s="4"/>
       <c r="Q113" s="4"/>
-      <c r="R113" s="4" t="s">
-        <v>613</v>
-      </c>
-      <c r="S113" s="8" t="s">
-        <v>614</v>
-      </c>
+      <c r="R113" s="4"/>
+      <c r="S113" s="4"/>
       <c r="T113" s="4"/>
       <c r="U113" s="4"/>
     </row>
-    <row r="114" spans="1:21" ht="130" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
-        <v>615</v>
+        <v>609</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>319</v>
+        <v>82</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="G114" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H114" s="4" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="I114" s="4" t="s">
-        <v>616</v>
+        <v>610</v>
       </c>
       <c r="J114" s="4"/>
       <c r="K114" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L114" s="4" t="s">
+      <c r="L114" s="8"/>
+      <c r="M114" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="N114" s="8"/>
+      <c r="O114" s="4"/>
+      <c r="P114" s="4"/>
+      <c r="Q114" s="4"/>
+      <c r="R114" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="S114" s="8" t="s">
+        <v>612</v>
+      </c>
+      <c r="T114" s="4"/>
+      <c r="U114" s="4"/>
+    </row>
+    <row r="115" spans="1:21" ht="130" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
+        <v>613</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="G115" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="H115" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="I115" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="J115" s="4"/>
+      <c r="K115" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L115" s="4" t="s">
+        <v>615</v>
+      </c>
+      <c r="M115" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="N115" s="4"/>
+      <c r="O115" s="6" t="s">
         <v>617</v>
       </c>
-      <c r="M114" s="4" t="s">
+      <c r="P115" s="6"/>
+      <c r="Q115" s="4" t="s">
         <v>618</v>
       </c>
-      <c r="N114" s="4"/>
-      <c r="O114" s="6" t="s">
+      <c r="R115" s="4" t="s">
         <v>619</v>
       </c>
-      <c r="P114" s="6"/>
-      <c r="Q114" s="4" t="s">
+      <c r="S115" s="8" t="s">
         <v>620</v>
       </c>
-      <c r="R114" s="4" t="s">
+      <c r="T115" s="4" t="s">
         <v>621</v>
       </c>
-      <c r="S114" s="8" t="s">
+      <c r="U115" s="4"/>
+    </row>
+    <row r="116" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
         <v>622</v>
       </c>
-      <c r="T114" s="4" t="s">
+      <c r="B116" s="2" t="s">
         <v>623</v>
       </c>
-      <c r="U114" s="4"/>
-    </row>
-    <row r="115" spans="1:21" ht="68" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="1" t="s">
+      <c r="D116" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="G116" s="3" t="s">
         <v>624</v>
       </c>
-      <c r="B115" s="2" t="s">
+      <c r="H116" s="10" t="s">
         <v>625</v>
       </c>
-      <c r="D115" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G115" s="3" t="s">
+      <c r="I116" s="10" t="s">
         <v>626</v>
       </c>
-      <c r="H115" s="10" t="s">
-        <v>627</v>
-      </c>
-      <c r="I115" s="10" t="s">
-        <v>628</v>
-      </c>
-      <c r="J115" s="10"/>
-      <c r="K115" s="4"/>
-      <c r="L115" s="4"/>
-      <c r="M115" s="4"/>
-      <c r="N115" s="4"/>
-      <c r="O115" s="4"/>
-      <c r="P115" s="4"/>
-      <c r="Q115" s="4"/>
-      <c r="R115" s="4" t="s">
-        <v>629</v>
-      </c>
-      <c r="S115" s="4"/>
-      <c r="T115" s="4"/>
-      <c r="U115" s="4"/>
-    </row>
-    <row r="116" spans="1:21" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="1" t="s">
-        <v>630</v>
-      </c>
-      <c r="D116" s="2">
-        <v>3</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G116" s="3" t="s">
-        <v>626</v>
-      </c>
-      <c r="H116" s="4" t="s">
-        <v>277</v>
-      </c>
-      <c r="I116" s="4" t="s">
-        <v>631</v>
-      </c>
-      <c r="J116" s="4"/>
-      <c r="K116" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L116" s="8"/>
-      <c r="M116" s="8" t="s">
-        <v>632</v>
-      </c>
+      <c r="J116" s="10"/>
+      <c r="K116" s="4"/>
+      <c r="L116" s="4"/>
+      <c r="M116" s="4"/>
       <c r="N116" s="4"/>
       <c r="O116" s="4"/>
       <c r="P116" s="4"/>
       <c r="Q116" s="4"/>
-      <c r="R116" s="14" t="s">
-        <v>633</v>
-      </c>
-      <c r="S116" s="4" t="s">
-        <v>634</v>
-      </c>
+      <c r="R116" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="S116" s="4"/>
       <c r="T116" s="4"/>
       <c r="U116" s="4"/>
     </row>
-    <row r="117" spans="1:21" ht="153" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:21" ht="54" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
-        <v>635</v>
+        <v>628</v>
       </c>
       <c r="D117" s="2">
         <v>3</v>
@@ -7897,182 +7889,189 @@
         <v>92</v>
       </c>
       <c r="G117" s="3" t="s">
-        <v>534</v>
+        <v>624</v>
       </c>
       <c r="H117" s="4" t="s">
         <v>277</v>
       </c>
       <c r="I117" s="4" t="s">
-        <v>636</v>
+        <v>629</v>
       </c>
       <c r="J117" s="4"/>
       <c r="K117" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L117" s="8" t="s">
-        <v>637</v>
-      </c>
+      <c r="L117" s="8"/>
       <c r="M117" s="8" t="s">
-        <v>638</v>
-      </c>
-      <c r="N117" s="8"/>
+        <v>630</v>
+      </c>
+      <c r="N117" s="4"/>
       <c r="O117" s="4"/>
       <c r="P117" s="4"/>
-      <c r="Q117" s="6"/>
-      <c r="R117" s="4" t="s">
-        <v>633</v>
+      <c r="Q117" s="4"/>
+      <c r="R117" s="14" t="s">
+        <v>631</v>
       </c>
       <c r="S117" s="4" t="s">
-        <v>639</v>
+        <v>632</v>
       </c>
       <c r="T117" s="4"/>
       <c r="U117" s="4"/>
     </row>
-    <row r="118" spans="1:21" ht="221" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:21" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
-        <v>640</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>39</v>
+        <v>633</v>
+      </c>
+      <c r="D118" s="2">
+        <v>3</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="G118" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H118" s="4" t="s">
         <v>277</v>
       </c>
       <c r="I118" s="4" t="s">
-        <v>641</v>
+        <v>634</v>
       </c>
       <c r="J118" s="4"/>
       <c r="K118" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L118" s="8" t="s">
-        <v>642</v>
+        <v>635</v>
       </c>
       <c r="M118" s="8" t="s">
-        <v>643</v>
+        <v>636</v>
       </c>
       <c r="N118" s="8"/>
-      <c r="O118" s="6" t="s">
-        <v>644</v>
-      </c>
-      <c r="P118" s="6"/>
-      <c r="Q118" s="4"/>
+      <c r="O118" s="4"/>
+      <c r="P118" s="4"/>
+      <c r="Q118" s="6"/>
       <c r="R118" s="4" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="S118" s="4" t="s">
-        <v>645</v>
+        <v>637</v>
       </c>
       <c r="T118" s="4"/>
       <c r="U118" s="4"/>
     </row>
-    <row r="119" spans="1:21" ht="204" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:21" ht="221" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="D119" s="2">
-        <v>3</v>
-      </c>
-      <c r="F119" s="2" t="s">
-        <v>92</v>
+        <v>638</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="G119" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H119" s="4" t="s">
         <v>277</v>
       </c>
       <c r="I119" s="4" t="s">
-        <v>647</v>
+        <v>639</v>
       </c>
       <c r="J119" s="4"/>
       <c r="K119" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L119" s="8" t="s">
-        <v>648</v>
+        <v>640</v>
       </c>
       <c r="M119" s="8" t="s">
-        <v>649</v>
-      </c>
-      <c r="N119" s="26" t="s">
-        <v>302</v>
-      </c>
+        <v>641</v>
+      </c>
+      <c r="N119" s="8"/>
       <c r="O119" s="6" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="P119" s="6"/>
       <c r="Q119" s="4"/>
-      <c r="R119" s="8" t="s">
-        <v>650</v>
-      </c>
-      <c r="S119" s="8" t="s">
-        <v>651</v>
+      <c r="R119" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="S119" s="4" t="s">
+        <v>643</v>
       </c>
       <c r="T119" s="4"/>
       <c r="U119" s="4"/>
     </row>
-    <row r="120" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
-        <v>652</v>
-      </c>
-      <c r="D120" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G120" s="20" t="s">
-        <v>534</v>
+        <v>644</v>
+      </c>
+      <c r="D120" s="2">
+        <v>3</v>
+      </c>
+      <c r="F120" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="G120" s="3" t="s">
+        <v>532</v>
       </c>
       <c r="H120" s="4" t="s">
-        <v>207</v>
+        <v>277</v>
       </c>
       <c r="I120" s="4" t="s">
-        <v>653</v>
+        <v>645</v>
       </c>
       <c r="J120" s="4"/>
       <c r="K120" s="4" t="s">
-        <v>654</v>
-      </c>
-      <c r="L120" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="M120" s="8"/>
-      <c r="N120" s="8"/>
-      <c r="O120" s="4"/>
-      <c r="P120" s="4"/>
+        <v>25</v>
+      </c>
+      <c r="L120" s="8" t="s">
+        <v>646</v>
+      </c>
+      <c r="M120" s="8" t="s">
+        <v>647</v>
+      </c>
+      <c r="N120" s="26" t="s">
+        <v>302</v>
+      </c>
+      <c r="O120" s="6" t="s">
+        <v>642</v>
+      </c>
+      <c r="P120" s="6"/>
       <c r="Q120" s="4"/>
-      <c r="R120" s="4"/>
-      <c r="S120" s="4"/>
+      <c r="R120" s="8" t="s">
+        <v>648</v>
+      </c>
+      <c r="S120" s="8" t="s">
+        <v>649</v>
+      </c>
       <c r="T120" s="4"/>
       <c r="U120" s="4"/>
     </row>
     <row r="121" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="D121" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G121" s="20" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H121" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="I121" s="8" t="s">
-        <v>656</v>
-      </c>
-      <c r="J121" s="8"/>
+      <c r="I121" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="J121" s="4"/>
       <c r="K121" s="4" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="L121" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="M121" s="4"/>
-      <c r="N121" s="4"/>
+      <c r="M121" s="8"/>
+      <c r="N121" s="8"/>
       <c r="O121" s="4"/>
       <c r="P121" s="4"/>
       <c r="Q121" s="4"/>
@@ -8083,31 +8082,31 @@
     </row>
     <row r="122" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
-        <v>657</v>
+        <v>653</v>
       </c>
       <c r="D122" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G122" s="20" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H122" s="4" t="s">
         <v>207</v>
       </c>
       <c r="I122" s="8" t="s">
-        <v>658</v>
+        <v>654</v>
       </c>
       <c r="J122" s="8"/>
       <c r="K122" s="4" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="L122" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="M122" s="8"/>
-      <c r="N122" s="8"/>
-      <c r="O122" s="6"/>
-      <c r="P122" s="6"/>
+      <c r="M122" s="4"/>
+      <c r="N122" s="4"/>
+      <c r="O122" s="4"/>
+      <c r="P122" s="4"/>
       <c r="Q122" s="4"/>
       <c r="R122" s="4"/>
       <c r="S122" s="4"/>
@@ -8116,102 +8115,96 @@
     </row>
     <row r="123" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
-        <v>659</v>
+        <v>655</v>
       </c>
       <c r="D123" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G123" s="20" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H123" s="4" t="s">
         <v>207</v>
       </c>
       <c r="I123" s="8" t="s">
-        <v>660</v>
+        <v>656</v>
       </c>
       <c r="J123" s="8"/>
       <c r="K123" s="4" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="L123" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="M123" s="4"/>
-      <c r="N123" s="4"/>
-      <c r="O123" s="4"/>
-      <c r="P123" s="4"/>
+      <c r="M123" s="8"/>
+      <c r="N123" s="8"/>
+      <c r="O123" s="6"/>
+      <c r="P123" s="6"/>
       <c r="Q123" s="4"/>
       <c r="R123" s="4"/>
       <c r="S123" s="4"/>
       <c r="T123" s="4"/>
       <c r="U123" s="4"/>
     </row>
-    <row r="124" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
-        <v>661</v>
-      </c>
-      <c r="B124" s="22" t="s">
-        <v>662</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>663</v>
+        <v>657</v>
       </c>
       <c r="D124" s="2" t="s">
         <v>39</v>
       </c>
       <c r="G124" s="20" t="s">
-        <v>626</v>
+        <v>532</v>
       </c>
       <c r="H124" s="4" t="s">
-        <v>664</v>
+        <v>207</v>
       </c>
       <c r="I124" s="8" t="s">
-        <v>665</v>
+        <v>658</v>
       </c>
       <c r="J124" s="8"/>
       <c r="K124" s="4" t="s">
-        <v>654</v>
-      </c>
-      <c r="L124" s="4"/>
+        <v>652</v>
+      </c>
+      <c r="L124" s="4" t="s">
+        <v>209</v>
+      </c>
       <c r="M124" s="4"/>
       <c r="N124" s="4"/>
       <c r="O124" s="4"/>
       <c r="P124" s="4"/>
       <c r="Q124" s="4"/>
-      <c r="R124" s="4" t="s">
-        <v>666</v>
-      </c>
+      <c r="R124" s="4"/>
       <c r="S124" s="4"/>
       <c r="T124" s="4"/>
-      <c r="U124" s="4" t="s">
-        <v>667</v>
-      </c>
-    </row>
-    <row r="125" spans="1:21" ht="81" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U124" s="4"/>
+    </row>
+    <row r="125" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
-        <v>668</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>669</v>
+        <v>659</v>
+      </c>
+      <c r="B125" s="22" t="s">
+        <v>660</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>670</v>
+        <v>661</v>
       </c>
       <c r="D125" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G125" s="3" t="s">
-        <v>534</v>
+      <c r="G125" s="20" t="s">
+        <v>624</v>
       </c>
       <c r="H125" s="4" t="s">
-        <v>627</v>
-      </c>
-      <c r="I125" s="4" t="s">
-        <v>671</v>
-      </c>
-      <c r="J125" s="4"/>
-      <c r="K125" s="4"/>
+        <v>662</v>
+      </c>
+      <c r="I125" s="8" t="s">
+        <v>663</v>
+      </c>
+      <c r="J125" s="8"/>
+      <c r="K125" s="4" t="s">
+        <v>652</v>
+      </c>
       <c r="L125" s="4"/>
       <c r="M125" s="4"/>
       <c r="N125" s="4"/>
@@ -8219,70 +8212,77 @@
       <c r="P125" s="4"/>
       <c r="Q125" s="4"/>
       <c r="R125" s="4" t="s">
-        <v>672</v>
+        <v>664</v>
       </c>
       <c r="S125" s="4"/>
       <c r="T125" s="4"/>
-      <c r="U125" s="4"/>
-    </row>
-    <row r="126" spans="1:21" ht="65" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U125" s="4" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="126" spans="1:21" ht="81" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
-        <v>673</v>
-      </c>
-      <c r="D126" s="2">
-        <v>3</v>
-      </c>
-      <c r="F126" s="2" t="s">
-        <v>314</v>
+        <v>666</v>
+      </c>
+      <c r="B126" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="D126" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="G126" s="3" t="s">
-        <v>534</v>
+        <v>532</v>
       </c>
       <c r="H126" s="4" t="s">
-        <v>277</v>
+        <v>625</v>
       </c>
       <c r="I126" s="4" t="s">
-        <v>674</v>
+        <v>669</v>
       </c>
       <c r="J126" s="4"/>
-      <c r="K126" s="4" t="s">
-        <v>654</v>
-      </c>
-      <c r="L126" s="8" t="s">
-        <v>675</v>
-      </c>
+      <c r="K126" s="4"/>
+      <c r="L126" s="4"/>
       <c r="M126" s="4"/>
       <c r="N126" s="4"/>
       <c r="O126" s="4"/>
       <c r="P126" s="4"/>
       <c r="Q126" s="4"/>
-      <c r="R126" s="4"/>
+      <c r="R126" s="4" t="s">
+        <v>670</v>
+      </c>
       <c r="S126" s="4"/>
       <c r="T126" s="4"/>
       <c r="U126" s="4"/>
     </row>
-    <row r="127" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:21" ht="65" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
-        <v>676</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>677</v>
-      </c>
-      <c r="D127" s="2" t="s">
-        <v>39</v>
+        <v>671</v>
+      </c>
+      <c r="D127" s="2">
+        <v>3</v>
+      </c>
+      <c r="F127" s="2" t="s">
+        <v>314</v>
       </c>
       <c r="G127" s="3" t="s">
-        <v>626</v>
-      </c>
-      <c r="H127" s="10" t="s">
-        <v>627</v>
-      </c>
-      <c r="I127" s="10" t="s">
-        <v>678</v>
-      </c>
-      <c r="J127" s="10"/>
-      <c r="K127" s="4"/>
-      <c r="L127" s="4"/>
+        <v>532</v>
+      </c>
+      <c r="H127" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="I127" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="J127" s="4"/>
+      <c r="K127" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="L127" s="8" t="s">
+        <v>673</v>
+      </c>
       <c r="M127" s="4"/>
       <c r="N127" s="4"/>
       <c r="O127" s="4"/>
@@ -8293,229 +8293,214 @@
       <c r="T127" s="4"/>
       <c r="U127" s="4"/>
     </row>
-    <row r="128" spans="1:21" ht="94" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
-        <v>679</v>
+        <v>674</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="D128" s="2">
-        <v>3</v>
+        <v>675</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="G128" s="3" t="s">
-        <v>538</v>
+        <v>624</v>
       </c>
       <c r="H128" s="10" t="s">
-        <v>681</v>
+        <v>625</v>
       </c>
       <c r="I128" s="10" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="J128" s="10"/>
       <c r="K128" s="4"/>
-      <c r="L128" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="M128" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="N128" s="6"/>
-      <c r="O128" s="6" t="s">
-        <v>540</v>
-      </c>
-      <c r="P128" s="6"/>
+      <c r="L128" s="4"/>
+      <c r="M128" s="4"/>
+      <c r="N128" s="4"/>
+      <c r="O128" s="4"/>
+      <c r="P128" s="4"/>
       <c r="Q128" s="4"/>
-      <c r="R128" s="4" t="s">
-        <v>683</v>
-      </c>
-      <c r="S128" s="8" t="s">
-        <v>684</v>
-      </c>
+      <c r="R128" s="4"/>
+      <c r="S128" s="4"/>
       <c r="T128" s="4"/>
       <c r="U128" s="4"/>
     </row>
-    <row r="129" spans="1:21" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:21" ht="94" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
-        <v>685</v>
+        <v>677</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>686</v>
+        <v>678</v>
       </c>
       <c r="D129" s="2">
         <v>3</v>
       </c>
       <c r="G129" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="H129" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="I129" s="10" t="s">
+        <v>680</v>
+      </c>
+      <c r="J129" s="10"/>
+      <c r="K129" s="4"/>
+      <c r="L129" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="M129" s="6" t="s">
         <v>538</v>
-      </c>
-      <c r="H129" s="10" t="s">
-        <v>681</v>
-      </c>
-      <c r="I129" s="4" t="s">
-        <v>687</v>
-      </c>
-      <c r="J129" s="4"/>
-      <c r="K129" s="4"/>
-      <c r="L129" s="4"/>
-      <c r="M129" s="6" t="s">
-        <v>688</v>
       </c>
       <c r="N129" s="6"/>
       <c r="O129" s="6" t="s">
-        <v>688</v>
+        <v>538</v>
       </c>
       <c r="P129" s="6"/>
       <c r="Q129" s="4"/>
       <c r="R129" s="4" t="s">
-        <v>689</v>
+        <v>681</v>
       </c>
       <c r="S129" s="8" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="T129" s="4"/>
       <c r="U129" s="4"/>
     </row>
-    <row r="130" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:21" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>691</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>246</v>
+        <v>684</v>
       </c>
       <c r="D130" s="2">
         <v>3</v>
       </c>
       <c r="G130" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H130" s="10" t="s">
-        <v>692</v>
-      </c>
-      <c r="I130" s="10" t="s">
-        <v>693</v>
-      </c>
-      <c r="J130" s="10"/>
-      <c r="K130" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L130" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="M130" s="4" t="s">
-        <v>694</v>
-      </c>
-      <c r="N130" s="4"/>
+        <v>679</v>
+      </c>
+      <c r="I130" s="4" t="s">
+        <v>685</v>
+      </c>
+      <c r="J130" s="4"/>
+      <c r="K130" s="4"/>
+      <c r="L130" s="4"/>
+      <c r="M130" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="N130" s="6"/>
       <c r="O130" s="6" t="s">
-        <v>256</v>
+        <v>686</v>
       </c>
       <c r="P130" s="6"/>
       <c r="Q130" s="4"/>
       <c r="R130" s="4" t="s">
-        <v>695</v>
+        <v>687</v>
       </c>
       <c r="S130" s="8" t="s">
-        <v>696</v>
+        <v>682</v>
       </c>
       <c r="T130" s="4"/>
       <c r="U130" s="4"/>
     </row>
-    <row r="131" spans="1:21" ht="136" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
-        <v>697</v>
+        <v>688</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>698</v>
+        <v>689</v>
+      </c>
+      <c r="C131" s="2" t="s">
+        <v>246</v>
       </c>
       <c r="D131" s="2">
         <v>3</v>
       </c>
-      <c r="F131" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="G131" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H131" s="4" t="s">
-        <v>699</v>
-      </c>
-      <c r="I131" s="4" t="s">
-        <v>700</v>
-      </c>
-      <c r="J131" s="4"/>
+        <v>536</v>
+      </c>
+      <c r="H131" s="10" t="s">
+        <v>690</v>
+      </c>
+      <c r="I131" s="10" t="s">
+        <v>691</v>
+      </c>
+      <c r="J131" s="10"/>
       <c r="K131" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L131" s="8"/>
-      <c r="M131" s="4"/>
+      <c r="L131" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="M131" s="4" t="s">
+        <v>692</v>
+      </c>
       <c r="N131" s="4"/>
-      <c r="O131" s="4"/>
-      <c r="P131" s="4"/>
+      <c r="O131" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="P131" s="6"/>
       <c r="Q131" s="4"/>
       <c r="R131" s="4" t="s">
-        <v>701</v>
-      </c>
-      <c r="S131" s="4" t="s">
-        <v>702</v>
+        <v>693</v>
+      </c>
+      <c r="S131" s="8" t="s">
+        <v>694</v>
       </c>
       <c r="T131" s="4"/>
       <c r="U131" s="4"/>
     </row>
-    <row r="132" spans="1:21" ht="187" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
-        <v>703</v>
-      </c>
-      <c r="B132" s="9" t="s">
-        <v>704</v>
-      </c>
-      <c r="C132" s="9"/>
-      <c r="D132" s="9">
+        <v>695</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="D132" s="2">
         <v>3</v>
       </c>
-      <c r="E132" s="9"/>
-      <c r="F132" s="9" t="s">
+      <c r="F132" s="2" t="s">
         <v>92</v>
       </c>
       <c r="G132" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H132" s="4" t="s">
-        <v>406</v>
-      </c>
-      <c r="I132" s="8" t="s">
-        <v>705</v>
-      </c>
-      <c r="J132" s="8"/>
+        <v>697</v>
+      </c>
+      <c r="I132" s="4" t="s">
+        <v>698</v>
+      </c>
+      <c r="J132" s="4"/>
       <c r="K132" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L132" s="8" t="s">
-        <v>706</v>
-      </c>
-      <c r="M132" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="N132" s="8"/>
+      <c r="L132" s="8"/>
+      <c r="M132" s="4"/>
+      <c r="N132" s="4"/>
       <c r="O132" s="4"/>
       <c r="P132" s="4"/>
       <c r="Q132" s="4"/>
       <c r="R132" s="4" t="s">
-        <v>707</v>
+        <v>699</v>
       </c>
       <c r="S132" s="4" t="s">
-        <v>708</v>
+        <v>700</v>
       </c>
       <c r="T132" s="4"/>
       <c r="U132" s="4"/>
     </row>
-    <row r="133" spans="1:21" ht="153" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
-        <v>709</v>
+        <v>701</v>
       </c>
       <c r="B133" s="9" t="s">
-        <v>710</v>
+        <v>702</v>
       </c>
       <c r="C133" s="9"/>
       <c r="D133" s="9">
@@ -8526,43 +8511,43 @@
         <v>92</v>
       </c>
       <c r="G133" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H133" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I133" s="8" t="s">
-        <v>711</v>
+        <v>703</v>
       </c>
       <c r="J133" s="8"/>
       <c r="K133" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L133" s="8" t="s">
-        <v>706</v>
-      </c>
-      <c r="M133" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="N133" s="11"/>
+        <v>704</v>
+      </c>
+      <c r="M133" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="N133" s="8"/>
       <c r="O133" s="4"/>
       <c r="P133" s="4"/>
       <c r="Q133" s="4"/>
       <c r="R133" s="4" t="s">
-        <v>712</v>
+        <v>705</v>
       </c>
       <c r="S133" s="4" t="s">
-        <v>713</v>
+        <v>706</v>
       </c>
       <c r="T133" s="4"/>
       <c r="U133" s="4"/>
     </row>
-    <row r="134" spans="1:21" ht="153" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:21" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
-        <v>697</v>
+        <v>707</v>
       </c>
       <c r="B134" s="9" t="s">
-        <v>698</v>
+        <v>708</v>
       </c>
       <c r="C134" s="9"/>
       <c r="D134" s="9">
@@ -8573,123 +8558,141 @@
         <v>92</v>
       </c>
       <c r="G134" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H134" s="4" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="I134" s="8" t="s">
-        <v>714</v>
+        <v>709</v>
       </c>
       <c r="J134" s="8"/>
       <c r="K134" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L134" s="8" t="s">
-        <v>706</v>
-      </c>
-      <c r="M134" s="4"/>
-      <c r="N134" s="4"/>
+        <v>704</v>
+      </c>
+      <c r="M134" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="N134" s="11"/>
       <c r="O134" s="4"/>
       <c r="P134" s="4"/>
       <c r="Q134" s="4"/>
       <c r="R134" s="4" t="s">
-        <v>715</v>
-      </c>
-      <c r="S134" s="8" t="s">
-        <v>702</v>
+        <v>710</v>
+      </c>
+      <c r="S134" s="4" t="s">
+        <v>711</v>
       </c>
       <c r="T134" s="4"/>
       <c r="U134" s="4"/>
     </row>
-    <row r="135" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:21" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
-        <v>716</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>717</v>
-      </c>
-      <c r="D135" s="2">
+        <v>695</v>
+      </c>
+      <c r="B135" s="9" t="s">
+        <v>696</v>
+      </c>
+      <c r="C135" s="9"/>
+      <c r="D135" s="9">
         <v>3</v>
       </c>
+      <c r="E135" s="9"/>
+      <c r="F135" s="9" t="s">
+        <v>92</v>
+      </c>
       <c r="G135" s="3" t="s">
-        <v>718</v>
+        <v>536</v>
       </c>
       <c r="H135" s="4" t="s">
-        <v>260</v>
+        <v>405</v>
       </c>
       <c r="I135" s="8" t="s">
-        <v>719</v>
+        <v>712</v>
       </c>
       <c r="J135" s="8"/>
       <c r="K135" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L135" s="23" t="s">
-        <v>706</v>
-      </c>
-      <c r="M135" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="N135" s="11"/>
+      <c r="L135" s="8" t="s">
+        <v>704</v>
+      </c>
+      <c r="M135" s="4"/>
+      <c r="N135" s="4"/>
       <c r="O135" s="4"/>
       <c r="P135" s="4"/>
       <c r="Q135" s="4"/>
       <c r="R135" s="4" t="s">
-        <v>720</v>
-      </c>
-      <c r="S135" s="4" t="s">
-        <v>721</v>
+        <v>713</v>
+      </c>
+      <c r="S135" s="8" t="s">
+        <v>700</v>
       </c>
       <c r="T135" s="4"/>
       <c r="U135" s="4"/>
     </row>
-    <row r="136" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:21" ht="204" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
-        <v>722</v>
-      </c>
-      <c r="D136" s="2" t="s">
-        <v>82</v>
+        <v>714</v>
+      </c>
+      <c r="B136" s="2" t="s">
+        <v>715</v>
+      </c>
+      <c r="D136" s="2">
+        <v>3</v>
       </c>
       <c r="G136" s="3" t="s">
-        <v>538</v>
+        <v>716</v>
       </c>
       <c r="H136" s="4" t="s">
-        <v>723</v>
-      </c>
-      <c r="I136" s="4" t="s">
-        <v>724</v>
-      </c>
-      <c r="J136" s="4"/>
-      <c r="K136" s="4"/>
-      <c r="L136" s="4"/>
-      <c r="M136" s="4"/>
-      <c r="N136" s="4"/>
+        <v>260</v>
+      </c>
+      <c r="I136" s="8" t="s">
+        <v>717</v>
+      </c>
+      <c r="J136" s="8"/>
+      <c r="K136" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L136" s="23" t="s">
+        <v>704</v>
+      </c>
+      <c r="M136" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="N136" s="11"/>
       <c r="O136" s="4"/>
       <c r="P136" s="4"/>
       <c r="Q136" s="4"/>
-      <c r="R136" s="4"/>
-      <c r="S136" s="8"/>
+      <c r="R136" s="4" t="s">
+        <v>718</v>
+      </c>
+      <c r="S136" s="4" t="s">
+        <v>719</v>
+      </c>
       <c r="T136" s="4"/>
       <c r="U136" s="4"/>
     </row>
-    <row r="137" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
-        <v>725</v>
+        <v>720</v>
       </c>
       <c r="D137" s="2" t="s">
         <v>82</v>
       </c>
       <c r="G137" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H137" s="10" t="s">
-        <v>723</v>
-      </c>
-      <c r="I137" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="J137" s="10"/>
+        <v>536</v>
+      </c>
+      <c r="H137" s="4" t="s">
+        <v>721</v>
+      </c>
+      <c r="I137" s="4" t="s">
+        <v>722</v>
+      </c>
+      <c r="J137" s="4"/>
       <c r="K137" s="4"/>
       <c r="L137" s="4"/>
       <c r="M137" s="4"/>
@@ -8697,31 +8700,26 @@
       <c r="O137" s="4"/>
       <c r="P137" s="4"/>
       <c r="Q137" s="4"/>
-      <c r="R137" s="4" t="s">
-        <v>726</v>
-      </c>
-      <c r="S137" s="4"/>
+      <c r="R137" s="4"/>
+      <c r="S137" s="8"/>
       <c r="T137" s="4"/>
       <c r="U137" s="4"/>
     </row>
-    <row r="138" spans="1:21" ht="85" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
-        <v>727</v>
-      </c>
-      <c r="B138" s="2" t="s">
-        <v>728</v>
+        <v>723</v>
       </c>
       <c r="D138" s="2" t="s">
         <v>82</v>
       </c>
       <c r="G138" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H138" s="10" t="s">
-        <v>729</v>
+        <v>721</v>
       </c>
       <c r="I138" s="10" t="s">
-        <v>730</v>
+        <v>83</v>
       </c>
       <c r="J138" s="10"/>
       <c r="K138" s="4"/>
@@ -8732,117 +8730,112 @@
       <c r="P138" s="4"/>
       <c r="Q138" s="4"/>
       <c r="R138" s="4" t="s">
-        <v>731</v>
+        <v>724</v>
       </c>
       <c r="S138" s="4"/>
       <c r="T138" s="4"/>
       <c r="U138" s="4"/>
     </row>
-    <row r="139" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:21" ht="85" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
-        <v>732</v>
+        <v>725</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>733</v>
-      </c>
-      <c r="D139" s="2">
-        <v>2</v>
+        <v>726</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="G139" s="3" t="s">
-        <v>538</v>
-      </c>
-      <c r="H139" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="I139" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="J139" s="4"/>
-      <c r="K139" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="L139" s="8" t="s">
-        <v>185</v>
-      </c>
-      <c r="M139" s="11" t="s">
-        <v>735</v>
-      </c>
-      <c r="N139" s="11"/>
+        <v>536</v>
+      </c>
+      <c r="H139" s="10" t="s">
+        <v>727</v>
+      </c>
+      <c r="I139" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="J139" s="10"/>
+      <c r="K139" s="4"/>
+      <c r="L139" s="4"/>
+      <c r="M139" s="4"/>
+      <c r="N139" s="4"/>
       <c r="O139" s="4"/>
       <c r="P139" s="4"/>
       <c r="Q139" s="4"/>
       <c r="R139" s="4" t="s">
-        <v>736</v>
-      </c>
-      <c r="S139" s="8" t="s">
-        <v>737</v>
-      </c>
+        <v>729</v>
+      </c>
+      <c r="S139" s="4"/>
       <c r="T139" s="4"/>
       <c r="U139" s="4"/>
     </row>
-    <row r="140" spans="1:21" ht="119" hidden="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
-        <v>738</v>
+        <v>730</v>
       </c>
       <c r="B140" s="2" t="s">
-        <v>739</v>
+        <v>731</v>
       </c>
       <c r="D140" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G140" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H140" s="10" t="s">
-        <v>260</v>
-      </c>
-      <c r="I140" s="10" t="s">
-        <v>740</v>
-      </c>
-      <c r="J140" s="10"/>
-      <c r="K140" s="4"/>
-      <c r="L140" s="4"/>
-      <c r="M140" s="4"/>
-      <c r="N140" s="4"/>
+        <v>536</v>
+      </c>
+      <c r="H140" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I140" s="4" t="s">
+        <v>732</v>
+      </c>
+      <c r="J140" s="4"/>
+      <c r="K140" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L140" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="M140" s="11" t="s">
+        <v>733</v>
+      </c>
+      <c r="N140" s="11"/>
       <c r="O140" s="4"/>
       <c r="P140" s="4"/>
       <c r="Q140" s="4"/>
-      <c r="R140" s="4"/>
-      <c r="S140" s="4"/>
+      <c r="R140" s="4" t="s">
+        <v>734</v>
+      </c>
+      <c r="S140" s="8" t="s">
+        <v>735</v>
+      </c>
       <c r="T140" s="4"/>
       <c r="U140" s="4"/>
     </row>
-    <row r="141" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:21" ht="119" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
-        <v>741</v>
+        <v>736</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>742</v>
-      </c>
-      <c r="C141" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="D141" s="2" t="s">
-        <v>82</v>
+        <v>737</v>
+      </c>
+      <c r="D141" s="2">
+        <v>1</v>
       </c>
       <c r="G141" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H141" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="I141" s="4" t="s">
-        <v>743</v>
-      </c>
-      <c r="J141" s="4"/>
-      <c r="K141" s="4" t="s">
-        <v>25</v>
-      </c>
+      <c r="H141" s="10" t="s">
+        <v>260</v>
+      </c>
+      <c r="I141" s="10" t="s">
+        <v>738</v>
+      </c>
+      <c r="J141" s="10"/>
+      <c r="K141" s="4"/>
       <c r="L141" s="4"/>
-      <c r="M141" s="8" t="s">
-        <v>607</v>
-      </c>
-      <c r="N141" s="8"/>
+      <c r="M141" s="4"/>
+      <c r="N141" s="4"/>
       <c r="O141" s="4"/>
       <c r="P141" s="4"/>
       <c r="Q141" s="4"/>
@@ -8851,24 +8844,27 @@
       <c r="T141" s="4"/>
       <c r="U141" s="4"/>
     </row>
-    <row r="142" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:21" ht="136" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
-        <v>744</v>
+        <v>739</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="D142" s="2">
-        <v>3</v>
-      </c>
-      <c r="G142" s="20" t="s">
-        <v>538</v>
+        <v>740</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>597</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G142" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="H142" s="4" t="s">
-        <v>175</v>
+        <v>74</v>
       </c>
       <c r="I142" s="4" t="s">
-        <v>745</v>
+        <v>741</v>
       </c>
       <c r="J142" s="4"/>
       <c r="K142" s="4" t="s">
@@ -8876,7 +8872,7 @@
       </c>
       <c r="L142" s="4"/>
       <c r="M142" s="8" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="N142" s="8"/>
       <c r="O142" s="4"/>
@@ -8887,372 +8883,419 @@
       <c r="T142" s="4"/>
       <c r="U142" s="4"/>
     </row>
-    <row r="143" spans="1:21" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:21" ht="51" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
-        <v>746</v>
+        <v>742</v>
+      </c>
+      <c r="B143" s="2" t="s">
+        <v>678</v>
       </c>
       <c r="D143" s="2">
         <v>3</v>
       </c>
-      <c r="F143" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="G143" s="3" t="s">
-        <v>538</v>
+      <c r="G143" s="20" t="s">
+        <v>536</v>
       </c>
       <c r="H143" s="4" t="s">
-        <v>747</v>
+        <v>175</v>
       </c>
       <c r="I143" s="4" t="s">
-        <v>748</v>
+        <v>743</v>
       </c>
       <c r="J143" s="4"/>
       <c r="K143" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L143" s="8" t="s">
-        <v>706</v>
-      </c>
-      <c r="M143" s="4"/>
-      <c r="N143" s="4"/>
+      <c r="L143" s="4"/>
+      <c r="M143" s="8" t="s">
+        <v>605</v>
+      </c>
+      <c r="N143" s="8"/>
       <c r="O143" s="4"/>
       <c r="P143" s="4"/>
       <c r="Q143" s="4"/>
-      <c r="R143" s="8" t="s">
-        <v>749</v>
-      </c>
-      <c r="S143" s="8" t="s">
-        <v>750</v>
-      </c>
+      <c r="R143" s="4"/>
+      <c r="S143" s="4"/>
       <c r="T143" s="4"/>
       <c r="U143" s="4"/>
     </row>
-    <row r="144" spans="1:21" ht="153" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:21" ht="80" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
-        <v>751</v>
+        <v>744</v>
       </c>
       <c r="D144" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F144" s="2" t="s">
         <v>92</v>
       </c>
       <c r="G144" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H144" s="4" t="s">
-        <v>565</v>
+        <v>745</v>
       </c>
       <c r="I144" s="4" t="s">
-        <v>752</v>
+        <v>746</v>
       </c>
       <c r="J144" s="4"/>
       <c r="K144" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L144" s="8" t="s">
-        <v>706</v>
-      </c>
-      <c r="M144" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="N144" s="8"/>
+        <v>704</v>
+      </c>
+      <c r="M144" s="4"/>
+      <c r="N144" s="4"/>
       <c r="O144" s="4"/>
       <c r="P144" s="4"/>
       <c r="Q144" s="4"/>
-      <c r="R144" s="4" t="s">
-        <v>753</v>
-      </c>
-      <c r="S144" s="4" t="s">
-        <v>754</v>
+      <c r="R144" s="8" t="s">
+        <v>747</v>
+      </c>
+      <c r="S144" s="8" t="s">
+        <v>748</v>
       </c>
       <c r="T144" s="4"/>
       <c r="U144" s="4"/>
     </row>
-    <row r="145" spans="1:21" ht="221" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:21" ht="153" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
-        <v>755</v>
-      </c>
-      <c r="B145" s="2" t="s">
-        <v>756</v>
+        <v>749</v>
       </c>
       <c r="D145" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F145" s="2" t="s">
         <v>92</v>
       </c>
       <c r="G145" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H145" s="4" t="s">
-        <v>757</v>
+        <v>563</v>
       </c>
       <c r="I145" s="4" t="s">
-        <v>758</v>
+        <v>750</v>
       </c>
       <c r="J145" s="4"/>
       <c r="K145" s="4" t="s">
         <v>25</v>
       </c>
       <c r="L145" s="8" t="s">
-        <v>706</v>
-      </c>
-      <c r="M145" s="11" t="s">
+        <v>704</v>
+      </c>
+      <c r="M145" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="N145" s="11"/>
+      <c r="N145" s="8"/>
       <c r="O145" s="4"/>
       <c r="P145" s="4"/>
       <c r="Q145" s="4"/>
       <c r="R145" s="4" t="s">
-        <v>759</v>
-      </c>
-      <c r="S145" s="8" t="s">
-        <v>760</v>
+        <v>751</v>
+      </c>
+      <c r="S145" s="4" t="s">
+        <v>752</v>
       </c>
       <c r="T145" s="4"/>
       <c r="U145" s="4"/>
     </row>
-    <row r="146" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:21" ht="221" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
-        <v>761</v>
+        <v>753</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>762</v>
+        <v>754</v>
       </c>
       <c r="D146" s="2">
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>92</v>
       </c>
       <c r="G146" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H146" s="4" t="s">
-        <v>757</v>
+        <v>755</v>
       </c>
       <c r="I146" s="4" t="s">
-        <v>763</v>
+        <v>756</v>
       </c>
       <c r="J146" s="4"/>
       <c r="K146" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L146" s="11"/>
-      <c r="M146" s="4"/>
-      <c r="N146" s="4"/>
+      <c r="L146" s="8" t="s">
+        <v>704</v>
+      </c>
+      <c r="M146" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="N146" s="11"/>
       <c r="O146" s="4"/>
       <c r="P146" s="4"/>
       <c r="Q146" s="4"/>
       <c r="R146" s="4" t="s">
-        <v>764</v>
-      </c>
-      <c r="S146" s="4"/>
+        <v>757</v>
+      </c>
+      <c r="S146" s="8" t="s">
+        <v>758</v>
+      </c>
       <c r="T146" s="4"/>
       <c r="U146" s="4"/>
     </row>
-    <row r="147" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:21" ht="102" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
-        <v>765</v>
+        <v>759</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>766</v>
-      </c>
-      <c r="D147" s="2" t="s">
-        <v>82</v>
+        <v>760</v>
+      </c>
+      <c r="D147" s="2">
+        <v>1</v>
       </c>
       <c r="G147" s="3" t="s">
-        <v>538</v>
+        <v>536</v>
       </c>
       <c r="H147" s="4" t="s">
-        <v>767</v>
-      </c>
-      <c r="I147" s="8" t="s">
-        <v>768</v>
-      </c>
-      <c r="J147" s="8"/>
+        <v>755</v>
+      </c>
+      <c r="I147" s="4" t="s">
+        <v>761</v>
+      </c>
+      <c r="J147" s="4"/>
       <c r="K147" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="L147" s="4"/>
-      <c r="M147" s="4" t="s">
-        <v>769</v>
-      </c>
+      <c r="L147" s="11"/>
+      <c r="M147" s="4"/>
       <c r="N147" s="4"/>
       <c r="O147" s="4"/>
       <c r="P147" s="4"/>
       <c r="Q147" s="4"/>
       <c r="R147" s="4" t="s">
-        <v>770</v>
-      </c>
-      <c r="S147" s="8" t="s">
-        <v>771</v>
-      </c>
+        <v>762</v>
+      </c>
+      <c r="S147" s="4"/>
       <c r="T147" s="4"/>
       <c r="U147" s="4"/>
     </row>
-    <row r="148" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A148" s="5" t="s">
+    <row r="148" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A148" s="1" t="s">
+        <v>763</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>764</v>
+      </c>
+      <c r="D148" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="G148" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="H148" s="4" t="s">
+        <v>765</v>
+      </c>
+      <c r="I148" s="8" t="s">
+        <v>766</v>
+      </c>
+      <c r="J148" s="8"/>
+      <c r="K148" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="L148" s="4"/>
+      <c r="M148" s="4" t="s">
+        <v>767</v>
+      </c>
+      <c r="N148" s="4"/>
+      <c r="O148" s="4"/>
+      <c r="P148" s="4"/>
+      <c r="Q148" s="4"/>
+      <c r="R148" s="4" t="s">
+        <v>768</v>
+      </c>
+      <c r="S148" s="8" t="s">
+        <v>769</v>
+      </c>
+      <c r="T148" s="4"/>
+      <c r="U148" s="4"/>
+    </row>
+    <row r="149" spans="1:21" ht="170" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A149" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="D148" s="2" t="s">
+      <c r="D149" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="G149" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="I149" s="5" t="s">
+        <v>771</v>
+      </c>
+      <c r="L149" s="24" t="s">
+        <v>630</v>
+      </c>
+      <c r="M149" s="5" t="s">
         <v>772</v>
       </c>
-      <c r="G148" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="I148" s="5" t="s">
+      <c r="O149" s="5" t="s">
         <v>773</v>
       </c>
-      <c r="L148" s="24" t="s">
-        <v>632</v>
-      </c>
-      <c r="M148" s="5" t="s">
+      <c r="R149" s="24" t="s">
         <v>774</v>
       </c>
-      <c r="O148" s="5" t="s">
+      <c r="S149" s="24" t="s">
         <v>775</v>
       </c>
-      <c r="R148" s="24" t="s">
-        <v>776</v>
-      </c>
-      <c r="S148" s="24" t="s">
-        <v>777</v>
-      </c>
-    </row>
-    <row r="149" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="5" t="s">
-        <v>640</v>
-      </c>
-      <c r="G149" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="I149" s="5" t="s">
-        <v>778</v>
-      </c>
-      <c r="K149" s="5" t="s">
-        <v>779</v>
-      </c>
-      <c r="L149" s="24" t="s">
-        <v>632</v>
-      </c>
-      <c r="R149" s="24"/>
-      <c r="S149" s="24"/>
     </row>
     <row r="150" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="G150" s="5" t="s">
+        <v>532</v>
+      </c>
+      <c r="I150" s="5" t="s">
+        <v>776</v>
+      </c>
+      <c r="K150" s="5" t="s">
+        <v>777</v>
+      </c>
+      <c r="L150" s="24" t="s">
+        <v>630</v>
+      </c>
+      <c r="R150" s="24"/>
+      <c r="S150" s="24"/>
+    </row>
+    <row r="151" spans="1:21" ht="34" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A151" s="5" t="s">
         <v>289</v>
-      </c>
-      <c r="D150" s="2">
-        <v>1</v>
-      </c>
-      <c r="G150" s="5" t="s">
-        <v>276</v>
-      </c>
-      <c r="I150" s="5" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="151" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="5" t="s">
-        <v>781</v>
       </c>
       <c r="D151" s="2">
         <v>1</v>
       </c>
       <c r="G151" s="5" t="s">
+        <v>276</v>
+      </c>
+      <c r="I151" s="5" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="152" spans="1:21" ht="187" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A152" s="5" t="s">
+        <v>779</v>
+      </c>
+      <c r="D152" s="2">
+        <v>1</v>
+      </c>
+      <c r="G152" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="I151" s="5" t="s">
+      <c r="I152" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="M152" s="24" t="s">
+        <v>781</v>
+      </c>
+      <c r="O152" s="25" t="s">
         <v>782</v>
       </c>
-      <c r="M151" s="24" t="s">
+      <c r="R152" s="5" t="s">
         <v>783</v>
       </c>
-      <c r="O151" s="25" t="s">
+    </row>
+    <row r="154" spans="1:21" ht="64" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A154" s="5" t="s">
         <v>784</v>
       </c>
-      <c r="R151" s="5" t="s">
-        <v>785</v>
-      </c>
-    </row>
-    <row r="153" spans="1:21" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A153" s="5" t="s">
-        <v>786</v>
-      </c>
-      <c r="D153" s="2" t="s">
-        <v>772</v>
-      </c>
-      <c r="G153" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="I153" s="5" t="s">
-        <v>787</v>
-      </c>
-      <c r="M153" s="25" t="s">
-        <v>788</v>
-      </c>
-      <c r="N153" s="25" t="s">
-        <v>789</v>
-      </c>
-      <c r="O153" s="25" t="s">
-        <v>790</v>
-      </c>
-      <c r="P153" s="25" t="s">
-        <v>784</v>
-      </c>
-      <c r="R153" s="24" t="s">
-        <v>791</v>
-      </c>
-      <c r="S153" s="5" t="s">
-        <v>792</v>
-      </c>
-    </row>
-    <row r="154" spans="1:21" ht="323" x14ac:dyDescent="0.2">
-      <c r="A154" s="5" t="s">
-        <v>793</v>
-      </c>
       <c r="D154" s="2" t="s">
-        <v>772</v>
+        <v>770</v>
       </c>
       <c r="G154" s="5" t="s">
         <v>343</v>
       </c>
       <c r="I154" s="5" t="s">
+        <v>785</v>
+      </c>
+      <c r="M154" s="25" t="s">
+        <v>786</v>
+      </c>
+      <c r="N154" s="25" t="s">
+        <v>787</v>
+      </c>
+      <c r="O154" s="25" t="s">
+        <v>788</v>
+      </c>
+      <c r="P154" s="25" t="s">
+        <v>782</v>
+      </c>
+      <c r="R154" s="24" t="s">
+        <v>789</v>
+      </c>
+      <c r="S154" s="5" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="155" spans="1:21" ht="323" x14ac:dyDescent="0.2">
+      <c r="A155" s="5" t="s">
+        <v>791</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="G155" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="I155" s="5" t="s">
+        <v>792</v>
+      </c>
+      <c r="M155" s="24" t="s">
+        <v>793</v>
+      </c>
+      <c r="N155" s="24" t="s">
         <v>794</v>
       </c>
-      <c r="M154" s="24" t="s">
+      <c r="O155" s="25" t="s">
         <v>795</v>
       </c>
-      <c r="N154" s="24" t="s">
-        <v>796</v>
-      </c>
-      <c r="O154" s="25" t="s">
-        <v>797</v>
-      </c>
-      <c r="P154" s="25"/>
+      <c r="P155" s="25"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U151" xr:uid="{576F2231-92F9-2048-8A13-39208F3A7342}">
-    <filterColumn colId="5">
+  <autoFilter ref="A1:U152" xr:uid="{576F2231-92F9-2048-8A13-39208F3A7342}">
+    <filterColumn colId="0">
       <filters>
-        <filter val="Bangladesh, India, Vietnam"/>
-        <filter val="Operandum"/>
-        <filter val="Vietnam"/>
-        <filter val="Vietnam - on going"/>
+        <filter val="E_EXP_ER"/>
+        <filter val="ER_CON_1512"/>
+        <filter val="ER_CON2"/>
+        <filter val="ER_ECO1"/>
+        <filter val="ER_FUN"/>
+        <filter val="ER_POL_1421"/>
+        <filter val="ER_POL_1521"/>
+        <filter val="ER_POL1"/>
+        <filter val="ER_POL2"/>
+        <filter val="ER_POL3"/>
+        <filter val="ER_POL4"/>
+        <filter val="ER_RES1"/>
+        <filter val="ER_RES2"/>
+        <filter val="ER_WAT1"/>
+        <filter val="ER_WAT2"/>
       </filters>
     </filterColumn>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="M99" r:id="rId1" xr:uid="{8CFCE988-EA10-C14A-9A06-C07DBDF0C8BC}"/>
+    <hyperlink ref="M100" r:id="rId1" xr:uid="{8CFCE988-EA10-C14A-9A06-C07DBDF0C8BC}"/>
     <hyperlink ref="M13" r:id="rId2" xr:uid="{7E605DBE-7FC9-1445-A32B-280B41EF2547}"/>
     <hyperlink ref="M44" r:id="rId3" xr:uid="{4CF7D1E2-8FEE-B049-935A-6F79D88C34A6}"/>
     <hyperlink ref="M86" r:id="rId4" display="https://www.unep-wcmc.org/" xr:uid="{6A6039D3-C5E8-BF4A-AE7F-B5335EA2552E}"/>
-    <hyperlink ref="M87" r:id="rId5" xr:uid="{1C06E689-3C30-C94F-A379-B3BDC88FA856}"/>
-    <hyperlink ref="M88" r:id="rId6" xr:uid="{C44C5616-3EF5-5B4E-B225-E31A5E851ACF}"/>
+    <hyperlink ref="M88" r:id="rId5" xr:uid="{1C06E689-3C30-C94F-A379-B3BDC88FA856}"/>
+    <hyperlink ref="M89" r:id="rId6" xr:uid="{C44C5616-3EF5-5B4E-B225-E31A5E851ACF}"/>
     <hyperlink ref="M75" r:id="rId7" xr:uid="{0FB83E1A-B316-FF4A-B108-AF3D5B044C25}"/>
     <hyperlink ref="L59" r:id="rId8" xr:uid="{09ED0199-452F-3F4D-97D0-18DEA0D0F469}"/>
     <hyperlink ref="M67" r:id="rId9" xr:uid="{4AA0573E-1829-744C-BCFF-06423AF767E1}"/>
-    <hyperlink ref="O119" r:id="rId10" xr:uid="{80F41256-667B-664C-9315-321E8D7FBABE}"/>
+    <hyperlink ref="O120" r:id="rId10" xr:uid="{80F41256-667B-664C-9315-321E8D7FBABE}"/>
     <hyperlink ref="O86" r:id="rId11" xr:uid="{9DC6504E-1055-4446-A4D2-0E6AA278E8D8}"/>
     <hyperlink ref="O75" r:id="rId12" xr:uid="{71A72F8D-CEBD-F449-AC08-BA6BF1247202}"/>
     <hyperlink ref="Q75" r:id="rId13" xr:uid="{982801E2-0404-B841-ACF3-91FA1D432EA9}"/>
@@ -9260,10 +9303,10 @@
     <hyperlink ref="M42" r:id="rId15" xr:uid="{C5B1550C-2B6C-6145-9C2C-F98E9FE04AA6}"/>
     <hyperlink ref="M38" r:id="rId16" xr:uid="{3ECF9AB2-B759-5042-9E0F-02B0F3C0314B}"/>
     <hyperlink ref="M32" r:id="rId17" xr:uid="{8BDD5F26-887B-CA46-8E5D-7642F677371D}"/>
-    <hyperlink ref="M90" r:id="rId18" xr:uid="{DDBE6515-484E-3644-B9F3-7CF6B6146736}"/>
+    <hyperlink ref="M91" r:id="rId18" xr:uid="{DDBE6515-484E-3644-B9F3-7CF6B6146736}"/>
     <hyperlink ref="O52" r:id="rId19" display="https://global-flood-database.cloudtostreet.ai/" xr:uid="{BF8A90CD-5A7B-AA42-8976-3E3C232C3BAB}"/>
-    <hyperlink ref="O118" r:id="rId20" xr:uid="{8DA06D71-CE5E-7544-8115-F4497A758DE0}"/>
-    <hyperlink ref="O114" r:id="rId21" xr:uid="{06D043E2-D022-4244-81BC-DBE8A4B9BFFB}"/>
+    <hyperlink ref="O119" r:id="rId20" xr:uid="{8DA06D71-CE5E-7544-8115-F4497A758DE0}"/>
+    <hyperlink ref="O115" r:id="rId21" xr:uid="{06D043E2-D022-4244-81BC-DBE8A4B9BFFB}"/>
     <hyperlink ref="O26" r:id="rId22" xr:uid="{CF7E386D-D34B-A641-9DC2-69B7958246BE}"/>
     <hyperlink ref="O80" r:id="rId23" xr:uid="{A2E630E2-5178-2840-B91B-1149B03768B0}"/>
     <hyperlink ref="O82" r:id="rId24" xr:uid="{F4AB9DE9-493A-0449-8B06-3C173E170BBA}"/>
@@ -9274,11 +9317,11 @@
     <hyperlink ref="O76" r:id="rId29" xr:uid="{717C0B30-5ECB-5E46-977C-C389B66CD868}"/>
     <hyperlink ref="O3" r:id="rId30" xr:uid="{6D4583C8-D1A5-C340-A58C-3C5C510FDF58}"/>
     <hyperlink ref="M26" r:id="rId31" xr:uid="{F91BC954-2FAF-F444-A928-84A17756A4AB}"/>
-    <hyperlink ref="M128" r:id="rId32" location="data/SDGB " xr:uid="{C8D4A9BA-D77B-D644-BC24-870E4AB668C8}"/>
-    <hyperlink ref="O128" r:id="rId33" location="data/SDGB " xr:uid="{C2A592F9-BEF8-DA4D-969B-93476E6C2938}"/>
-    <hyperlink ref="M129" r:id="rId34" xr:uid="{DA8BE33E-B011-094C-AA32-F5B79EE68BBC}"/>
-    <hyperlink ref="O129" r:id="rId35" xr:uid="{9A478AD5-E05D-8143-B496-927ADDD08F61}"/>
-    <hyperlink ref="M95" r:id="rId36" location="data/SDGB " xr:uid="{2F7197B8-A69B-6F40-8F86-24B122825FD9}"/>
+    <hyperlink ref="M129" r:id="rId32" location="data/SDGB " xr:uid="{C8D4A9BA-D77B-D644-BC24-870E4AB668C8}"/>
+    <hyperlink ref="O129" r:id="rId33" location="data/SDGB " xr:uid="{C2A592F9-BEF8-DA4D-969B-93476E6C2938}"/>
+    <hyperlink ref="M130" r:id="rId34" xr:uid="{DA8BE33E-B011-094C-AA32-F5B79EE68BBC}"/>
+    <hyperlink ref="O130" r:id="rId35" xr:uid="{9A478AD5-E05D-8143-B496-927ADDD08F61}"/>
+    <hyperlink ref="M96" r:id="rId36" location="data/SDGB " xr:uid="{2F7197B8-A69B-6F40-8F86-24B122825FD9}"/>
     <hyperlink ref="M7" r:id="rId37" xr:uid="{2AB4F7EA-6CC9-EF41-BA6A-7244E3EC3268}"/>
     <hyperlink ref="M4" r:id="rId38" display="https://unstats.un.org/sdgs/dataportal / / " xr:uid="{CFDB6AD6-B44F-E348-8BF9-1D0C1C17846D}"/>
     <hyperlink ref="O4" r:id="rId39" xr:uid="{06FB1F7C-99E9-6845-AF46-EBF85CE08BD6}"/>
@@ -9286,24 +9329,24 @@
     <hyperlink ref="O5" r:id="rId41" xr:uid="{7B1D9384-8E7D-0940-8ED8-6811E1089E4A}"/>
     <hyperlink ref="O6" r:id="rId42" xr:uid="{5A883D75-6DE1-7743-A106-BED94CB01403}"/>
     <hyperlink ref="M6" r:id="rId43" xr:uid="{49A0D79C-9623-E04E-90A0-70C931686A5D}"/>
-    <hyperlink ref="M97" r:id="rId44" xr:uid="{67E57890-CD21-8642-B957-DE579F98CD48}"/>
-    <hyperlink ref="M108" r:id="rId45" xr:uid="{094DF145-3A8D-9848-9893-5198344B0172}"/>
-    <hyperlink ref="O109" r:id="rId46" xr:uid="{197F2259-5D9F-0947-ADA1-8D13DA10B5A4}"/>
-    <hyperlink ref="M109" r:id="rId47" xr:uid="{1E286142-AE7D-0B43-A5AE-8B97DC7496E4}"/>
+    <hyperlink ref="M98" r:id="rId44" xr:uid="{67E57890-CD21-8642-B957-DE579F98CD48}"/>
+    <hyperlink ref="M109" r:id="rId45" xr:uid="{094DF145-3A8D-9848-9893-5198344B0172}"/>
+    <hyperlink ref="O110" r:id="rId46" xr:uid="{197F2259-5D9F-0947-ADA1-8D13DA10B5A4}"/>
+    <hyperlink ref="M110" r:id="rId47" xr:uid="{1E286142-AE7D-0B43-A5AE-8B97DC7496E4}"/>
     <hyperlink ref="M73" r:id="rId48" xr:uid="{303B49B3-DBA0-5544-A01F-EC9D682DF632}"/>
     <hyperlink ref="O73" r:id="rId49" xr:uid="{D89A4BCD-FEAE-E946-9FAE-CAAD87351813}"/>
     <hyperlink ref="M83" r:id="rId50" xr:uid="{133B2CBC-0022-4B4B-A8C3-EB9CC3464A63}"/>
     <hyperlink ref="M65" r:id="rId51" xr:uid="{3D29D4E9-7F0B-BD46-BD43-D50E1582FA5C}"/>
-    <hyperlink ref="O130" r:id="rId52" xr:uid="{FE66B1AE-25E5-1941-88AA-6F180FAF2F08}"/>
+    <hyperlink ref="O131" r:id="rId52" xr:uid="{FE66B1AE-25E5-1941-88AA-6F180FAF2F08}"/>
     <hyperlink ref="O44" r:id="rId53" xr:uid="{CD3A7A3F-C019-C14E-A6CE-72703AE59A6E}"/>
-    <hyperlink ref="O153" r:id="rId54" xr:uid="{63C8190A-9626-7E48-A836-82ECC2706751}"/>
-    <hyperlink ref="M153" r:id="rId55" xr:uid="{E9E1DBFB-9F21-1849-8B59-B4715B4A3BDD}"/>
-    <hyperlink ref="O154" r:id="rId56" xr:uid="{28C2B0B3-4772-E542-B419-0A3EB763659C}"/>
-    <hyperlink ref="N153" r:id="rId57" xr:uid="{2854BE3C-8847-C34F-9BF0-8A1BB92ECDE0}"/>
-    <hyperlink ref="P153" r:id="rId58" xr:uid="{291ED414-A2C8-154C-9B4E-FEB5C6275F0F}"/>
-    <hyperlink ref="O151" r:id="rId59" xr:uid="{D17BB223-5C6B-1F4D-BE64-F254BD5B4A27}"/>
+    <hyperlink ref="O154" r:id="rId54" xr:uid="{63C8190A-9626-7E48-A836-82ECC2706751}"/>
+    <hyperlink ref="M154" r:id="rId55" xr:uid="{E9E1DBFB-9F21-1849-8B59-B4715B4A3BDD}"/>
+    <hyperlink ref="O155" r:id="rId56" xr:uid="{28C2B0B3-4772-E542-B419-0A3EB763659C}"/>
+    <hyperlink ref="N154" r:id="rId57" xr:uid="{2854BE3C-8847-C34F-9BF0-8A1BB92ECDE0}"/>
+    <hyperlink ref="P154" r:id="rId58" xr:uid="{291ED414-A2C8-154C-9B4E-FEB5C6275F0F}"/>
+    <hyperlink ref="O152" r:id="rId59" xr:uid="{D17BB223-5C6B-1F4D-BE64-F254BD5B4A27}"/>
     <hyperlink ref="N52" r:id="rId60" xr:uid="{DF720B88-05E9-E048-9872-7C83EE0473D8}"/>
-    <hyperlink ref="N119" r:id="rId61" xr:uid="{81858DD3-4B4E-A243-91D7-D9F2D8EBD8DF}"/>
+    <hyperlink ref="N120" r:id="rId61" xr:uid="{81858DD3-4B4E-A243-91D7-D9F2D8EBD8DF}"/>
     <hyperlink ref="O56" r:id="rId62" xr:uid="{8FB81324-2595-7344-BA71-A9230B9D1D4B}"/>
     <hyperlink ref="N59" r:id="rId63" xr:uid="{4D80D5A6-E8C2-404B-B71F-594C7209EE5E}"/>
   </hyperlinks>

</xml_diff>